<commit_message>
Actualizacion automatica del mapa (2026-05-26 15:08:47)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R114"/>
+  <dimension ref="A1:R116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8349,7 +8349,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>813631418</t>
+        </is>
+      </c>
       <c r="H93" t="inlineStr">
         <is>
           <t>APLOMAR COLUMNA</t>
@@ -8431,7 +8435,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>813631419</t>
+        </is>
+      </c>
       <c r="H94" t="inlineStr">
         <is>
           <t>APLOMAR COLUMNA</t>
@@ -8509,7 +8517,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>813631455</t>
+        </is>
+      </c>
       <c r="H95" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -8591,7 +8603,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>813631875</t>
+        </is>
+      </c>
       <c r="H96" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -9465,7 +9481,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">10007 </t>
+          <t xml:space="preserve">9945 </t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -9475,7 +9491,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>CABEZON, JOSE LEON 3614</t>
+          <t>LACROZE, FEDERICO AV. 1938</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9518,24 +9534,24 @@
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>-58.515037</v>
+        <v>-58.440759</v>
       </c>
       <c r="N107" t="n">
-        <v>-34.589042</v>
+        <v>-34.565819</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9547,22 +9563,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">8734 </t>
+          <t xml:space="preserve">10007 </t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>ARISMENDI 2916</t>
+          <t>CABEZON, JOSE LEON 3614</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -9600,10 +9616,10 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>-58.479126</v>
+        <v>-58.515037</v>
       </c>
       <c r="N108" t="n">
-        <v>-34.586673</v>
+        <v>-34.589042</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -9617,7 +9633,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -9629,7 +9645,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">10037 </t>
+          <t xml:space="preserve">8726 </t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -9639,12 +9655,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>HERNANDARIAS 1957</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -9675,31 +9691,31 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L109" t="n">
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>-58.50158</v>
+        <v>-58.366665</v>
       </c>
       <c r="N109" t="n">
-        <v>-34.648954</v>
+        <v>-34.646956</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>CON-E</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -9711,7 +9727,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">10058 </t>
+          <t xml:space="preserve">8734 </t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -9721,12 +9737,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">OLIDEN 1187 </t>
+          <t>ARISMENDI 2916</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -9742,12 +9758,12 @@
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -9764,14 +9780,14 @@
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>-58.507509</v>
+        <v>-58.479126</v>
       </c>
       <c r="N110" t="n">
-        <v>-34.650225</v>
+        <v>-34.586673</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
@@ -9781,7 +9797,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>PAV-I</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -9793,7 +9809,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">10073 </t>
+          <t xml:space="preserve">10037 </t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -9803,12 +9819,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU 3464</t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -9824,12 +9840,12 @@
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -9839,17 +9855,17 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L111" t="n">
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>-58.511499</v>
+        <v>-58.50158</v>
       </c>
       <c r="N111" t="n">
-        <v>-34.603949</v>
+        <v>-34.648954</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -9863,7 +9879,7 @@
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>DEV-C</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -9875,7 +9891,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">10096 </t>
+          <t xml:space="preserve">10058 </t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -9885,12 +9901,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>RAMIREZ, CEFERINO, COMODORO 5402</t>
+          <t xml:space="preserve">OLIDEN 1187 </t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -9906,17 +9922,17 @@
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -9928,24 +9944,24 @@
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>-58.460409</v>
+        <v>-58.507509</v>
       </c>
       <c r="N112" t="n">
-        <v>-34.684521</v>
+        <v>-34.650225</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -9957,7 +9973,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">10097 </t>
+          <t xml:space="preserve">10073 </t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -9967,12 +9983,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>DESCALZI, NICOLAS 5404</t>
+          <t>GUALEGUAYCHU 3464</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -9988,12 +10004,12 @@
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -10010,24 +10026,24 @@
         <v>1</v>
       </c>
       <c r="M113" t="n">
-        <v>-58.463809</v>
+        <v>-58.511499</v>
       </c>
       <c r="N113" t="n">
-        <v>-34.68275</v>
+        <v>-34.603949</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>DEV-C</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10039,7 +10055,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">10151 </t>
+          <t xml:space="preserve">10096 </t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -10049,12 +10065,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>LAGUNA 1562</t>
+          <t>RAMIREZ, CEFERINO, COMODORO 5402</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -10070,49 +10086,213 @@
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>1</v>
+      </c>
+      <c r="M114" t="n">
+        <v>-58.460409</v>
+      </c>
+      <c r="N114" t="n">
+        <v>-34.684521</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10097 </t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>DESCALZI, NICOLAS 5404</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>DESMONTAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Desmonte</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L115" t="n">
+        <v>1</v>
+      </c>
+      <c r="M115" t="n">
+        <v>-58.463809</v>
+      </c>
+      <c r="N115" t="n">
+        <v>-34.68275</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10151 </t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>LAGUNA 1562</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
           <t>COLUMNA INCLINADA</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr">
+      <c r="I116" t="inlineStr">
         <is>
           <t>Aplomo</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr">
+      <c r="J116" t="inlineStr">
         <is>
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr">
+      <c r="K116" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="L114" t="n">
-        <v>1</v>
-      </c>
-      <c r="M114" t="n">
+      <c r="L116" t="n">
+        <v>1</v>
+      </c>
+      <c r="M116" t="n">
         <v>-58.467824</v>
       </c>
-      <c r="N114" t="n">
+      <c r="N116" t="n">
         <v>-34.649072</v>
       </c>
-      <c r="O114" t="inlineStr">
+      <c r="O116" t="inlineStr">
         <is>
           <t>Devoto</t>
         </is>
       </c>
-      <c r="P114" t="inlineStr">
+      <c r="P116" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="Q114" t="inlineStr">
+      <c r="Q116" t="inlineStr">
         <is>
           <t>PPT-N</t>
         </is>
       </c>
-      <c r="R114" t="inlineStr">
+      <c r="R116" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-27 13:41:19)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R97"/>
+  <dimension ref="A1:R91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4543,7 +4543,11 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>8882</t>
+        </is>
+      </c>
       <c r="B49" t="inlineStr">
         <is>
           <t>3/18/2026</t>
@@ -4551,508 +4555,524 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>GALLARDO, ANGEL AV. 1072</t>
+          <t>EL PROFETA DE LA PAMPA 4523</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>812879773</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L49" t="n">
+        <v>1</v>
+      </c>
+      <c r="M49" t="n">
+        <v>-58.477211</v>
+      </c>
+      <c r="N49" t="n">
+        <v>-34.652708</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>PAV-O</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>00239146</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>3/19/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>POLA 1104</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>812879780</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
+        <v>1</v>
+      </c>
+      <c r="M50" t="n">
+        <v>-58.50158</v>
+      </c>
+      <c r="N50" t="n">
+        <v>-34.648954</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>PAV-J</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7460 </t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>3/21/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>TERRADA 2720</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>812879976</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>RIENDA A PIQUE CORTADA</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Aplomo</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" t="n">
+        <v>-58.486103</v>
+      </c>
+      <c r="N51" t="n">
+        <v>-34.603895</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>NRA-P</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>00000609</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>3/21/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ZELADA 4402</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>812879764</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>812880445</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L49" t="n">
-        <v>1</v>
-      </c>
-      <c r="M49" t="n">
-        <v>-58.444908</v>
-      </c>
-      <c r="N49" t="n">
-        <v>-34.607205</v>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>ALM-O</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
+      <c r="L52" t="n">
+        <v>1</v>
+      </c>
+      <c r="M52" t="n">
+        <v>-58.48834</v>
+      </c>
+      <c r="N52" t="n">
+        <v>-34.641018</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>PCH-S</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2PCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11070617 </t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>3/28/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>FONROUGE 1697</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>812880729</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
+        <v>1</v>
+      </c>
+      <c r="M53" t="n">
+        <v>-58.496881</v>
+      </c>
+      <c r="N53" t="n">
+        <v>-34.653948</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>PAV-H</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>3/18/2026</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>GALLARDO, ANGEL AV. 1072</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>812879764</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">900009880510 </t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>GUTENBERG 4150</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>813046368</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>CAMBIAR POSTE POR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L50" t="n">
-        <v>1</v>
-      </c>
-      <c r="M50" t="n">
-        <v>-58.419576</v>
-      </c>
-      <c r="N50" t="n">
-        <v>-34.621289</v>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>ALM-A</t>
-        </is>
-      </c>
-      <c r="R50" t="inlineStr">
+      <c r="L54" t="n">
+        <v>1</v>
+      </c>
+      <c r="M54" t="n">
+        <v>-58.516791</v>
+      </c>
+      <c r="N54" t="n">
+        <v>-34.596662</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>PUE-P</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>3/18/2026</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>GALLARDO, ANGEL AV. 1072</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>812879764</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L51" t="n">
-        <v>1</v>
-      </c>
-      <c r="M51" t="n">
-        <v>-58.430568</v>
-      </c>
-      <c r="N51" t="n">
-        <v>-34.599485</v>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>CLI-N</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>3/18/2026</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>GALLARDO, ANGEL AV. 1072</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>812879764</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L52" t="n">
-        <v>1</v>
-      </c>
-      <c r="M52" t="n">
-        <v>-58.437499</v>
-      </c>
-      <c r="N52" t="n">
-        <v>-34.578324</v>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>ATH-B</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>3/18/2026</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>GALLARDO, ANGEL AV. 1072</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>812879764</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L53" t="n">
-        <v>1</v>
-      </c>
-      <c r="M53" t="n">
-        <v>-58.435547</v>
-      </c>
-      <c r="N53" t="n">
-        <v>-34.576622</v>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>ATH-B</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>3/18/2026</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>GALLARDO, ANGEL AV. 1072</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>812879764</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Reubicar columna y rienda, Angel Gallardo 1072 a 1084</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L54" t="n">
-        <v>1</v>
-      </c>
-      <c r="M54" t="n">
-        <v>-58.373629</v>
-      </c>
-      <c r="N54" t="n">
-        <v>-34.64417</v>
-      </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>San Telmo</t>
-        </is>
-      </c>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>CON-A</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>ARATO-25058.AF.1CON</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>8882</t>
+          <t>S00373014</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>3/18/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>EL PROFETA DE LA PAMPA 4523</t>
+          <t>BYRON 150</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5067,7 +5087,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>812879773</t>
+          <t>813046780</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5082,7 +5102,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -5094,10 +5114,10 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.477211</v>
+        <v>-58.501659</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.652708</v>
+        <v>-34.63959</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -5111,7 +5131,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>PAV-O</t>
+          <t>PAV-F</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5123,22 +5143,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>00239146</t>
+          <t>8819</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>3/19/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>CUENCA 2082</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5153,17 +5173,17 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>812879780</t>
+          <t>813046813</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>NORMALIZAR RIENDA A PIQUE</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Tensor</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -5173,17 +5193,17 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L56" t="n">
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.50158</v>
+        <v>-58.487454</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.648954</v>
+        <v>-34.610697</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -5197,7 +5217,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>NRA-O</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5209,22 +5229,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">7460 </t>
+          <t>8831</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>TERRADA 2720</t>
+          <t>FLORES VENACIO GRAL 4567</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5239,17 +5259,17 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>812879976</t>
+          <t>813046868</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>RIENDA A PIQUE CORTADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -5259,31 +5279,27 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L57" t="n">
-        <v>0</v>
-      </c>
-      <c r="M57" t="n">
-        <v>-58.486103</v>
-      </c>
-      <c r="N57" t="n">
-        <v>-34.603895</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>No clasificado, consultar con mantenimiento</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5295,17 +5311,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>00000609</t>
+          <t>8832</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ZELADA 4402</t>
+          <t>SANTO TOME 6674</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5325,7 +5341,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>812880445</t>
+          <t>813046870</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5352,10 +5368,10 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.48834</v>
+        <v>-58.528021</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.641018</v>
+        <v>-34.627813</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5369,34 +5385,34 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>DEV-O</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">11070617 </t>
+          <t>8686</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>3/28/2026</t>
+          <t>4/11/2026</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>FONROUGE 1697</t>
+          <t>CERVANTES 650</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -5411,7 +5427,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>812880729</t>
+          <t>813047531</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -5438,10 +5454,10 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.496881</v>
+        <v>-58.497176</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.653948</v>
+        <v>-34.631131</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -5455,25 +5471,29 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>DEV-M</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009880510 </t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr"/>
+          <t>S00391032</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>4/11/2026</t>
+        </is>
+      </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>GUTENBERG 4150</t>
+          <t>MARISCAL SOLANO LOPEZ 3312</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5493,12 +5513,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>813046368</t>
+          <t>813047700</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
+          <t>DESMONTAR POSTE Y COLOCAR COLUMNA</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5520,10 +5540,10 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.516791</v>
+        <v>-58.501067</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.596662</v>
+        <v>-34.596916</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -5537,7 +5557,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PUE-P</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5549,22 +5569,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S00373014</t>
+          <t>S00400580</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/14/2026</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>BYRON 150</t>
+          <t>BORDABEHERE, ENZO 2802</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5579,12 +5599,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>813046780</t>
+          <t>813304660</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR POSTE DE MADERA POR COLUMNA</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5606,14 +5626,14 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.501659</v>
+        <v>-58.480405</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.63959</v>
+        <v>-34.600087</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -5623,7 +5643,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PAV-F</t>
+          <t>PUE-A</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5635,17 +5655,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>8819</t>
+          <t>HALVAREZ</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CUENCA 2082</t>
+          <t>ASUNCION 3719</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -5665,17 +5685,17 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>813046813</t>
+          <t>813304738</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>NORMALIZAR RIENDA A PIQUE</t>
+          <t>DESMONTAR POSTE Y NORMALIZAR RED</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Tensor</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -5692,14 +5712,14 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.487454</v>
+        <v>-58.5078</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.610697</v>
+        <v>-34.598769</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -5709,7 +5729,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>NRA-O</t>
+          <t>PUE-P</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5721,22 +5741,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>8831</t>
+          <t>GG00035</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>FLORES VENACIO GRAL 4567</t>
+          <t>FIGUEROA, D. APOLINARIO, CORONEL 1793</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5751,7 +5771,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>813046868</t>
+          <t>813304912</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5761,7 +5781,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -5777,21 +5797,25 @@
       <c r="L63" t="n">
         <v>1</v>
       </c>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
+      <c r="M63" t="n">
+        <v>-58.461005</v>
+      </c>
+      <c r="N63" t="n">
+        <v>-34.613152</v>
+      </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>No clasificado, consultar con mantenimiento</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>NRA-J</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5803,17 +5827,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>8832</t>
+          <t>8954</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SANTO TOME 6674</t>
+          <t>FLORES, VENANCIO, GRAL. 4550</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5833,7 +5857,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>813046870</t>
+          <t>813350688</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5860,10 +5884,10 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.528021</v>
+        <v>-58.490636</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.627813</v>
+        <v>-34.634459</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -5877,34 +5901,34 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>DEV-O</t>
+          <t>DEV-M</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>8686</t>
+          <t>8994</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CERVANTES 650</t>
+          <t>COSQUIN 296</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5919,7 +5943,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>813047531</t>
+          <t>813350808</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5946,10 +5970,10 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.497176</v>
+        <v>-58.523272</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.631131</v>
+        <v>-34.642619</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -5963,29 +5987,29 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>DEV-M</t>
+          <t>PAV-C</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>S00391032</t>
+          <t>9022</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>MARISCAL SOLANO LOPEZ 3312</t>
+          <t xml:space="preserve">MAGARIÑOS CERVANTES, A. 2072 </t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -6005,12 +6029,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>813047700</t>
+          <t>813352594</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y COLOCAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6032,10 +6056,10 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.501067</v>
+        <v>-58.46936</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.596916</v>
+        <v>-34.60805</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -6049,7 +6073,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6061,22 +6085,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S00400580</t>
+          <t>S00463265</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>4/14/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>BORDABEHERE, ENZO 2802</t>
+          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6091,12 +6115,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>813304660</t>
+          <t>813353208</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE DE MADERA POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6118,14 +6142,14 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.480405</v>
+        <v>-58.508425</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.600087</v>
+        <v>-34.653353</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6135,7 +6159,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PUE-A</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6147,17 +6171,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>HALVAREZ</t>
+          <t xml:space="preserve">9070 </t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ASUNCION 3719</t>
+          <t>MORAN, PEDRO 3941</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -6177,17 +6201,17 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>813304738</t>
+          <t>813631418</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y NORMALIZAR RED</t>
+          <t>APLOMAR COLUMNA</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -6204,10 +6228,10 @@
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.5078</v>
+        <v>-58.509815</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.598769</v>
+        <v>-34.601072</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -6233,17 +6257,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GG00035</t>
+          <t xml:space="preserve">9071 </t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>FIGUEROA, D. APOLINARIO, CORONEL 1793</t>
+          <t xml:space="preserve">NAVARRO 4193 </t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -6263,12 +6287,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>813304912</t>
+          <t>813631419</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>APLOMAR COLUMNA</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6281,23 +6305,19 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K69" t="inlineStr"/>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.461005</v>
+        <v>-58.511033</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.613152</v>
+        <v>-34.604149</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -6307,7 +6327,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NRA-J</t>
+          <t>DEV-C</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6319,22 +6339,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>8954</t>
+          <t>S00488557</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>4/21/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 4550</t>
+          <t>COSQUIN 296</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6349,7 +6369,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>813350688</t>
+          <t>813631455</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -6376,10 +6396,10 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.490636</v>
+        <v>-58.523272</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.634459</v>
+        <v>-34.642619</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -6393,34 +6413,34 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>DEV-M</t>
+          <t>PAV-C</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>8994</t>
+          <t>S00369718</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>4/21/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COSQUIN 296</t>
+          <t>FLORES, VENANCIO, GRAL. 4568</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -6435,7 +6455,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>813350808</t>
+          <t>813631875</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -6462,10 +6482,10 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.523272</v>
+        <v>-58.490942</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.642619</v>
+        <v>-34.634502</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6479,29 +6499,29 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>PAV-C</t>
+          <t>DEV-M</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>9022</t>
+          <t xml:space="preserve">9139 </t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGARIÑOS CERVANTES, A. 2072 </t>
+          <t>MOSCONI GENERAL AV. 3327</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -6519,11 +6539,7 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>813352594</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -6548,10 +6564,10 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.46936</v>
+        <v>-58.508028</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.60805</v>
+        <v>-34.589722</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -6565,7 +6581,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>PUE-N</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6577,22 +6593,22 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S00463265</t>
+          <t>S00497584</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
+          <t>SOLANO LOPEZ, F., MARISCAL 3280</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6605,19 +6621,15 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>813353208</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t xml:space="preserve">DESMONTAR POSTE MADERA </t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -6634,14 +6646,14 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.508425</v>
+        <v>-58.500541</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.653353</v>
+        <v>-34.596596</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -6651,7 +6663,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6663,22 +6675,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">9070 </t>
+          <t>S00510491</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MORAN, PEDRO 3941</t>
+          <t>BRUIX AV. 4472</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6691,19 +6703,15 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>813631418</t>
-        </is>
-      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>APLOMAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -6720,14 +6728,14 @@
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.509815</v>
+        <v>-58.487496</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.601072</v>
+        <v>-34.646926</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -6737,7 +6745,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PUE-P</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6749,17 +6757,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">9071 </t>
+          <t xml:space="preserve">900009976210 </t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAVARRO 4193 </t>
+          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -6777,19 +6785,15 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>813631419</t>
-        </is>
-      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>APLOMAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -6797,19 +6801,23 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L75" t="n">
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.511033</v>
+        <v>-58.477456</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.604149</v>
+        <v>-34.614971</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -6819,7 +6827,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>DEV-C</t>
+          <t>NRA-M</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -6831,22 +6839,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>S00488557</t>
+          <t>9938</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>COSQUIN 296</t>
+          <t>QUESADA 5060</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6859,19 +6867,15 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>813631455</t>
-        </is>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -6888,14 +6892,14 @@
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.523272</v>
+        <v>-58.489366</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.642619</v>
+        <v>-34.568013</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
@@ -6905,7 +6909,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PAV-C</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6917,22 +6921,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>S00369718</t>
+          <t xml:space="preserve">9939 </t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 4568</t>
+          <t xml:space="preserve">QUESADA 5090 </t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -6945,19 +6949,15 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>813631875</t>
-        </is>
-      </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -6974,14 +6974,14 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.490942</v>
+        <v>-58.489722</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.634502</v>
+        <v>-34.568197</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -6991,19 +6991,19 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>DEV-M</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">9139 </t>
+          <t xml:space="preserve">9940 </t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>MOSCONI GENERAL AV. 3327</t>
+          <t>QUESADA 5210</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7034,12 +7034,12 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -7056,10 +7056,10 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.508028</v>
+        <v>-58.491219</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.589722</v>
+        <v>-34.568967</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -7073,7 +7073,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>PUE-N</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7085,7 +7085,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>S00497584</t>
+          <t xml:space="preserve">9942 </t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SOLANO LOPEZ, F., MARISCAL 3280</t>
+          <t>CAPDEVILA 3057</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7116,12 +7116,12 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t xml:space="preserve">DESMONTAR POSTE MADERA </t>
+          <t>COLUMN INCLINADA</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -7138,10 +7138,10 @@
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.500541</v>
+        <v>-58.490684</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.596596</v>
+        <v>-34.569213</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -7155,7 +7155,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7167,7 +7167,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>S00510491</t>
+          <t xml:space="preserve">9943 </t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7177,12 +7177,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>BRUIX AV. 4472</t>
+          <t>TRIUNVIRATO AV. 5359</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7198,12 +7198,12 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -7220,14 +7220,14 @@
         <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.487496</v>
+        <v>-58.491694</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.646926</v>
+        <v>-34.569911</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7237,7 +7237,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7249,7 +7249,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009976210 </t>
+          <t xml:space="preserve">9945 </t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7259,12 +7259,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
+          <t>LACROZE, FEDERICO AV. 1938</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7302,24 +7302,24 @@
         <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>-58.477456</v>
+        <v>-58.440759</v>
       </c>
       <c r="N81" t="n">
-        <v>-34.614971</v>
+        <v>-34.565819</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>NRA-M</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7331,7 +7331,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>9938</t>
+          <t xml:space="preserve">10007 </t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -7341,7 +7341,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>QUESADA 5060</t>
+          <t>CABEZON, JOSE LEON 3614</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7362,12 +7362,12 @@
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -7384,10 +7384,10 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>-58.489366</v>
+        <v>-58.515037</v>
       </c>
       <c r="N82" t="n">
-        <v>-34.568013</v>
+        <v>-34.589042</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
@@ -7401,7 +7401,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7413,22 +7413,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">9939 </t>
+          <t xml:space="preserve">8726 </t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">QUESADA 5090 </t>
+          <t>HERNANDARIAS 1957</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -7444,12 +7444,12 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -7466,24 +7466,24 @@
         <v>1</v>
       </c>
       <c r="M83" t="n">
-        <v>-58.489722</v>
+        <v>-58.366665</v>
       </c>
       <c r="N83" t="n">
-        <v>-34.568197</v>
+        <v>-34.646956</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>CON-E</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -7495,22 +7495,22 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">9940 </t>
+          <t xml:space="preserve">8734 </t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>QUESADA 5210</t>
+          <t>ARISMENDI 2916</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -7526,12 +7526,12 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -7548,10 +7548,10 @@
         <v>1</v>
       </c>
       <c r="M84" t="n">
-        <v>-58.491219</v>
+        <v>-58.479126</v>
       </c>
       <c r="N84" t="n">
-        <v>-34.568967</v>
+        <v>-34.586673</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -7577,22 +7577,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">9942 </t>
+          <t xml:space="preserve">10037 </t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CAPDEVILA 3057</t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -7608,12 +7608,12 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>COLUMN INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -7623,21 +7623,21 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L85" t="n">
         <v>1</v>
       </c>
       <c r="M85" t="n">
-        <v>-58.490684</v>
+        <v>-58.50158</v>
       </c>
       <c r="N85" t="n">
-        <v>-34.569213</v>
+        <v>-34.648954</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7659,22 +7659,22 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">9943 </t>
+          <t xml:space="preserve">10058 </t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>TRIUNVIRATO AV. 5359</t>
+          <t xml:space="preserve">OLIDEN 1187 </t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -7712,14 +7712,14 @@
         <v>1</v>
       </c>
       <c r="M86" t="n">
-        <v>-58.491694</v>
+        <v>-58.507509</v>
       </c>
       <c r="N86" t="n">
-        <v>-34.569911</v>
+        <v>-34.650225</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -7741,22 +7741,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">9945 </t>
+          <t xml:space="preserve">10073 </t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 1938</t>
+          <t>GUALEGUAYCHU 3464</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -7772,12 +7772,12 @@
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -7794,24 +7794,24 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>-58.440759</v>
+        <v>-58.511499</v>
       </c>
       <c r="N87" t="n">
-        <v>-34.565819</v>
+        <v>-34.603949</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>DEV-C</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -7823,22 +7823,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">10007 </t>
+          <t xml:space="preserve">10097 </t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CABEZON, JOSE LEON 3614</t>
+          <t>DESCALZI, NICOLAS 5404</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -7854,12 +7854,12 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -7876,24 +7876,24 @@
         <v>1</v>
       </c>
       <c r="M88" t="n">
-        <v>-58.515037</v>
+        <v>-58.463809</v>
       </c>
       <c r="N88" t="n">
-        <v>-34.589042</v>
+        <v>-34.68275</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -7905,7 +7905,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">8726 </t>
+          <t xml:space="preserve">10151 </t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -7915,12 +7915,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>HERNANDARIAS 1957</t>
+          <t>LAGUNA 1562</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -7936,12 +7936,12 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -7951,31 +7951,31 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L89" t="n">
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.366665</v>
+        <v>-58.467824</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.646956</v>
+        <v>-34.649072</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>CON-E</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -7987,17 +7987,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">8734 </t>
+          <t>-4992</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ARISMENDI 2916</t>
+          <t>BEYROUTH 4992</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -8018,7 +8018,7 @@
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>REALIZAR CAMBIO DE POSTE POR COLUMNA</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -8037,17 +8037,17 @@
         </is>
       </c>
       <c r="L90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M90" t="n">
-        <v>-58.479126</v>
+        <v>-58.502223</v>
       </c>
       <c r="N90" t="n">
-        <v>-34.586673</v>
+        <v>-34.626887</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -8057,7 +8057,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>DEV-H</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8069,22 +8069,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">10037 </t>
+          <t>-4926</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>BEYROUTH 4926</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -8100,7 +8100,7 @@
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR POSTE POR COLUMNA</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -8115,17 +8115,17 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L91" t="n">
         <v>1</v>
       </c>
       <c r="M91" t="n">
-        <v>-58.50158</v>
+        <v>-58.501459</v>
       </c>
       <c r="N91" t="n">
-        <v>-34.648954</v>
+        <v>-34.626196</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -8139,502 +8139,10 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>DEV-H</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10058 </t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OLIDEN 1187 </t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>COLUMNA INCLINADA</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>Aplomo</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L92" t="n">
-        <v>1</v>
-      </c>
-      <c r="M92" t="n">
-        <v>-58.507509</v>
-      </c>
-      <c r="N92" t="n">
-        <v>-34.650225</v>
-      </c>
-      <c r="O92" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P92" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q92" t="inlineStr">
-        <is>
-          <t>PAV-I</t>
-        </is>
-      </c>
-      <c r="R92" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10073 </t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>GUALEGUAYCHU 3464</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>COLUMNA INCLINADA</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>Aplomo</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L93" t="n">
-        <v>1</v>
-      </c>
-      <c r="M93" t="n">
-        <v>-58.511499</v>
-      </c>
-      <c r="N93" t="n">
-        <v>-34.603949</v>
-      </c>
-      <c r="O93" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P93" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q93" t="inlineStr">
-        <is>
-          <t>DEV-C</t>
-        </is>
-      </c>
-      <c r="R93" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10097 </t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>DESCALZI, NICOLAS 5404</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>DESMONTAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>Desmonte</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L94" t="n">
-        <v>1</v>
-      </c>
-      <c r="M94" t="n">
-        <v>-58.463809</v>
-      </c>
-      <c r="N94" t="n">
-        <v>-34.68275</v>
-      </c>
-      <c r="O94" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P94" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q94" t="inlineStr">
-        <is>
-          <t>PAV-U</t>
-        </is>
-      </c>
-      <c r="R94" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10151 </t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>LAGUNA 1562</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>COLUMNA INCLINADA</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>Aplomo</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="L95" t="n">
-        <v>1</v>
-      </c>
-      <c r="M95" t="n">
-        <v>-58.467824</v>
-      </c>
-      <c r="N95" t="n">
-        <v>-34.649072</v>
-      </c>
-      <c r="O95" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P95" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q95" t="inlineStr">
-        <is>
-          <t>PPT-N</t>
-        </is>
-      </c>
-      <c r="R95" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>-4992</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>5/26/2026</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>BEYROUTH 4992</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>REALIZAR CAMBIO DE POSTE POR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L96" t="n">
-        <v>0</v>
-      </c>
-      <c r="M96" t="n">
-        <v>-58.502223</v>
-      </c>
-      <c r="N96" t="n">
-        <v>-34.626887</v>
-      </c>
-      <c r="O96" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P96" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q96" t="inlineStr">
-        <is>
-          <t>DEV-H</t>
-        </is>
-      </c>
-      <c r="R96" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>-4926</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>5/26/2026</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>BEYROUTH 4926</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J97" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L97" t="n">
-        <v>1</v>
-      </c>
-      <c r="M97" t="n">
-        <v>-58.501459</v>
-      </c>
-      <c r="N97" t="n">
-        <v>-34.626196</v>
-      </c>
-      <c r="O97" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P97" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q97" t="inlineStr">
-        <is>
-          <t>DEV-H</t>
-        </is>
-      </c>
-      <c r="R97" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-28 07:55:14)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R91"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5569,7 +5569,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S00400580</t>
+          <t>S00387253</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5579,12 +5579,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>BORDABEHERE, ENZO 2802</t>
+          <t>DIAZ, CESAR, GRAL. 4881</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5599,12 +5599,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>813304660</t>
+          <t>813304416</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE DE MADERA POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5626,14 +5626,14 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.480405</v>
+        <v>-58.49779</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.600087</v>
+        <v>-34.627626</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PUE-A</t>
+          <t>DEV-I</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5655,17 +5655,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>HALVAREZ</t>
+          <t>S00400580</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/14/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ASUNCION 3719</t>
+          <t>BORDABEHERE, ENZO 2802</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -5685,12 +5685,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>813304738</t>
+          <t>813304660</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y NORMALIZAR RED</t>
+          <t>CAMBIAR POSTE DE MADERA POR COLUMNA</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5712,10 +5712,10 @@
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.5078</v>
+        <v>-58.480405</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.598769</v>
+        <v>-34.600087</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PUE-P</t>
+          <t>PUE-A</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5741,7 +5741,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>GG00035</t>
+          <t>HALVAREZ</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>FIGUEROA, D. APOLINARIO, CORONEL 1793</t>
+          <t>ASUNCION 3719</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -5771,17 +5771,17 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>813304912</t>
+          <t>813304738</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE Y NORMALIZAR RED</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -5798,10 +5798,10 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.461005</v>
+        <v>-58.5078</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.613152</v>
+        <v>-34.598769</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -5815,7 +5815,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>NRA-J</t>
+          <t>PUE-P</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5827,22 +5827,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>8954</t>
+          <t>GG00035</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>4/21/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 4550</t>
+          <t>FIGUEROA, D. APOLINARIO, CORONEL 1793</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5857,7 +5857,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>813350688</t>
+          <t>813304912</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -5884,14 +5884,14 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.490636</v>
+        <v>-58.461005</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.634459</v>
+        <v>-34.613152</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -5901,19 +5901,19 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>DEV-M</t>
+          <t>NRA-J</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>8994</t>
+          <t>8954</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -5923,12 +5923,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>COSQUIN 296</t>
+          <t>FLORES, VENANCIO, GRAL. 4550</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>813350808</t>
+          <t>813350688</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5970,10 +5970,10 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.523272</v>
+        <v>-58.490636</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.642619</v>
+        <v>-34.634459</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -5987,34 +5987,34 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>PAV-C</t>
+          <t>DEV-M</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>9022</t>
+          <t>8994</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGARIÑOS CERVANTES, A. 2072 </t>
+          <t>COSQUIN 296</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>813352594</t>
+          <t>813350808</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -6056,14 +6056,14 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.46936</v>
+        <v>-58.523272</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.60805</v>
+        <v>-34.642619</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>PAV-C</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6085,7 +6085,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S00463265</t>
+          <t>9022</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6095,12 +6095,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
+          <t xml:space="preserve">MAGARIÑOS CERVANTES, A. 2072 </t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6115,7 +6115,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>813353208</t>
+          <t>813352594</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -6142,14 +6142,14 @@
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.508425</v>
+        <v>-58.46936</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.653353</v>
+        <v>-34.60805</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -6159,7 +6159,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6171,22 +6171,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">9070 </t>
+          <t>S00463265</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>MORAN, PEDRO 3941</t>
+          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6201,17 +6201,17 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>813631418</t>
+          <t>813353208</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>APLOMAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -6228,14 +6228,14 @@
         <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.509815</v>
+        <v>-58.508425</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.601072</v>
+        <v>-34.653353</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>PUE-P</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">9071 </t>
+          <t xml:space="preserve">9070 </t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6267,7 +6267,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAVARRO 4193 </t>
+          <t>MORAN, PEDRO 3941</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>813631419</t>
+          <t>813631418</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -6305,19 +6305,23 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.511033</v>
+        <v>-58.509815</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.604149</v>
+        <v>-34.601072</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -6327,7 +6331,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>DEV-C</t>
+          <t>PUE-P</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6339,7 +6343,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S00488557</t>
+          <t xml:space="preserve">9071 </t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -6349,12 +6353,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>COSQUIN 296</t>
+          <t xml:space="preserve">NAVARRO 4193 </t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6369,17 +6373,17 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>813631455</t>
+          <t>813631419</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>APLOMAR COLUMNA</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -6387,19 +6391,15 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+      <c r="K70" t="inlineStr"/>
       <c r="L70" t="n">
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.523272</v>
+        <v>-58.511033</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.642619</v>
+        <v>-34.604149</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -6413,7 +6413,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>PAV-C</t>
+          <t>DEV-C</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6425,22 +6425,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S00369718</t>
+          <t>S00488557</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 4568</t>
+          <t>COSQUIN 296</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -6455,7 +6455,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>813631875</t>
+          <t>813631455</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -6482,10 +6482,10 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.490942</v>
+        <v>-58.523272</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.634502</v>
+        <v>-34.642619</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6499,34 +6499,34 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>DEV-M</t>
+          <t>PAV-C</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">9139 </t>
+          <t>S00369718</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>MOSCONI GENERAL AV. 3327</t>
+          <t>FLORES, VENANCIO, GRAL. 4568</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -6539,7 +6539,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>813631875</t>
+        </is>
+      </c>
       <c r="H72" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -6564,14 +6568,14 @@
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.508028</v>
+        <v>-58.490942</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.589722</v>
+        <v>-34.634502</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
@@ -6581,19 +6585,19 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>PUE-N</t>
+          <t>DEV-M</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S00497584</t>
+          <t xml:space="preserve">9139 </t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6603,7 +6607,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SOLANO LOPEZ, F., MARISCAL 3280</t>
+          <t>MOSCONI GENERAL AV. 3327</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -6624,12 +6628,12 @@
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t xml:space="preserve">DESMONTAR POSTE MADERA </t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -6646,10 +6650,10 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.500541</v>
+        <v>-58.508028</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.596596</v>
+        <v>-34.589722</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -6663,7 +6667,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>PUE-N</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6675,7 +6679,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S00510491</t>
+          <t>S00497584</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6685,12 +6689,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>BRUIX AV. 4472</t>
+          <t>SOLANO LOPEZ, F., MARISCAL 3280</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6706,12 +6710,12 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t xml:space="preserve">DESMONTAR POSTE MADERA </t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -6728,14 +6732,14 @@
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.487496</v>
+        <v>-58.500541</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.646926</v>
+        <v>-34.596596</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -6745,7 +6749,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6757,7 +6761,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009976210 </t>
+          <t>S00510491</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -6767,12 +6771,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
+          <t>BRUIX AV. 4472</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -6810,14 +6814,14 @@
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.477456</v>
+        <v>-58.487496</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.614971</v>
+        <v>-34.646926</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -6827,7 +6831,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>NRA-M</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -6839,7 +6843,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>9938</t>
+          <t xml:space="preserve">900009976210 </t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -6849,7 +6853,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>QUESADA 5060</t>
+          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -6870,12 +6874,12 @@
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -6892,10 +6896,10 @@
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.489366</v>
+        <v>-58.477456</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.568013</v>
+        <v>-34.614971</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -6909,7 +6913,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>NRA-M</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6921,7 +6925,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">9939 </t>
+          <t>9938</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -6931,7 +6935,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">QUESADA 5090 </t>
+          <t>QUESADA 5060</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -6974,10 +6978,10 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.489722</v>
+        <v>-58.489366</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.568197</v>
+        <v>-34.568013</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -7003,7 +7007,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">9940 </t>
+          <t xml:space="preserve">9939 </t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -7013,7 +7017,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>QUESADA 5210</t>
+          <t xml:space="preserve">QUESADA 5090 </t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7056,10 +7060,10 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.491219</v>
+        <v>-58.489722</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.568967</v>
+        <v>-34.568197</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -7085,7 +7089,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">9942 </t>
+          <t xml:space="preserve">9940 </t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -7095,7 +7099,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CAPDEVILA 3057</t>
+          <t>QUESADA 5210</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7116,7 +7120,7 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>COLUMN INCLINADA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7138,10 +7142,10 @@
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>-58.490684</v>
+        <v>-58.491219</v>
       </c>
       <c r="N79" t="n">
-        <v>-34.569213</v>
+        <v>-34.568967</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -7167,7 +7171,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">9943 </t>
+          <t xml:space="preserve">9942 </t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7177,7 +7181,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TRIUNVIRATO AV. 5359</t>
+          <t>CAPDEVILA 3057</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7198,7 +7202,7 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>COLUMN INCLINADA</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7220,10 +7224,10 @@
         <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>-58.491694</v>
+        <v>-58.490684</v>
       </c>
       <c r="N80" t="n">
-        <v>-34.569911</v>
+        <v>-34.569213</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
@@ -7249,7 +7253,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">9945 </t>
+          <t xml:space="preserve">9943 </t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7259,12 +7263,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 1938</t>
+          <t>TRIUNVIRATO AV. 5359</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7280,12 +7284,12 @@
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -7302,24 +7306,24 @@
         <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>-58.440759</v>
+        <v>-58.491694</v>
       </c>
       <c r="N81" t="n">
-        <v>-34.565819</v>
+        <v>-34.569911</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7331,7 +7335,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">10007 </t>
+          <t xml:space="preserve">9945 </t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -7341,12 +7345,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CABEZON, JOSE LEON 3614</t>
+          <t>LACROZE, FEDERICO AV. 1938</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7384,24 +7388,24 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>-58.515037</v>
+        <v>-58.440759</v>
       </c>
       <c r="N82" t="n">
-        <v>-34.589042</v>
+        <v>-34.565819</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>BLO-L</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7413,22 +7417,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">8726 </t>
+          <t xml:space="preserve">10007 </t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HERNANDARIAS 1957</t>
+          <t>CABEZON, JOSE LEON 3614</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -7466,24 +7470,24 @@
         <v>1</v>
       </c>
       <c r="M83" t="n">
-        <v>-58.366665</v>
+        <v>-58.515037</v>
       </c>
       <c r="N83" t="n">
-        <v>-34.646956</v>
+        <v>-34.589042</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>CON-E</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -7495,7 +7499,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">8734 </t>
+          <t xml:space="preserve">8726 </t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -7505,12 +7509,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ARISMENDI 2916</t>
+          <t>HERNANDARIAS 1957</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -7548,24 +7552,24 @@
         <v>1</v>
       </c>
       <c r="M84" t="n">
-        <v>-58.479126</v>
+        <v>-58.366665</v>
       </c>
       <c r="N84" t="n">
-        <v>-34.586673</v>
+        <v>-34.646956</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>CON-E</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -7577,7 +7581,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">10037 </t>
+          <t xml:space="preserve">8734 </t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7587,12 +7591,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>ARISMENDI 2916</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -7623,21 +7627,21 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L85" t="n">
         <v>1</v>
       </c>
       <c r="M85" t="n">
-        <v>-58.50158</v>
+        <v>-58.479126</v>
       </c>
       <c r="N85" t="n">
-        <v>-34.648954</v>
+        <v>-34.586673</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
@@ -7647,7 +7651,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7659,7 +7663,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">10058 </t>
+          <t xml:space="preserve">10037 </t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7669,7 +7673,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">OLIDEN 1187 </t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7690,12 +7694,12 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -7705,17 +7709,17 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L86" t="n">
         <v>1</v>
       </c>
       <c r="M86" t="n">
-        <v>-58.507509</v>
+        <v>-58.50158</v>
       </c>
       <c r="N86" t="n">
-        <v>-34.650225</v>
+        <v>-34.648954</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -7729,7 +7733,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>PAV-I</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -7741,7 +7745,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">10073 </t>
+          <t xml:space="preserve">10058 </t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7751,12 +7755,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU 3464</t>
+          <t xml:space="preserve">OLIDEN 1187 </t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -7794,10 +7798,10 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>-58.511499</v>
+        <v>-58.507509</v>
       </c>
       <c r="N87" t="n">
-        <v>-34.603949</v>
+        <v>-34.650225</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -7811,7 +7815,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>DEV-C</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -7823,7 +7827,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">10097 </t>
+          <t xml:space="preserve">10073 </t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -7833,12 +7837,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>DESCALZI, NICOLAS 5404</t>
+          <t>GUALEGUAYCHU 3464</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -7854,12 +7858,12 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -7876,24 +7880,24 @@
         <v>1</v>
       </c>
       <c r="M88" t="n">
-        <v>-58.463809</v>
+        <v>-58.511499</v>
       </c>
       <c r="N88" t="n">
-        <v>-34.68275</v>
+        <v>-34.603949</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>DEV-C</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -7905,7 +7909,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">10151 </t>
+          <t xml:space="preserve">10097 </t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -7915,7 +7919,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>LAGUNA 1562</t>
+          <t>DESCALZI, NICOLAS 5404</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -7936,12 +7940,12 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>DESMONTAR COLUMNA</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -7951,31 +7955,31 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L89" t="n">
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.467824</v>
+        <v>-58.463809</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.649072</v>
+        <v>-34.68275</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -7987,22 +7991,22 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>-4992</t>
+          <t xml:space="preserve">10151 </t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>BEYROUTH 4992</t>
+          <t>LAGUNA 1562</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -8018,12 +8022,12 @@
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>REALIZAR CAMBIO DE POSTE POR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -8033,17 +8037,17 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M90" t="n">
-        <v>-58.502223</v>
+        <v>-58.467824</v>
       </c>
       <c r="N90" t="n">
-        <v>-34.626887</v>
+        <v>-34.649072</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
@@ -8057,7 +8061,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>DEV-H</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8069,7 +8073,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>-4926</t>
+          <t>-4992</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -8079,7 +8083,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>BEYROUTH 4926</t>
+          <t>BEYROUTH 4992</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8100,49 +8104,131 @@
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
+          <t>REALIZAR CAMBIO DE POSTE POR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
+        <v>-58.502223</v>
+      </c>
+      <c r="N91" t="n">
+        <v>-34.626887</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>DEV-H</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>-4926</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>5/26/2026</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>BEYROUTH 4926</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
           <t>CAMBIAR POSTE POR COLUMNA</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
+      <c r="I92" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr">
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L91" t="n">
-        <v>1</v>
-      </c>
-      <c r="M91" t="n">
+      <c r="L92" t="n">
+        <v>1</v>
+      </c>
+      <c r="M92" t="n">
         <v>-58.501459</v>
       </c>
-      <c r="N91" t="n">
+      <c r="N92" t="n">
         <v>-34.626196</v>
       </c>
-      <c r="O91" t="inlineStr">
+      <c r="O92" t="inlineStr">
         <is>
           <t>Devoto</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q91" t="inlineStr">
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
         <is>
           <t>DEV-H</t>
         </is>
       </c>
-      <c r="R91" t="inlineStr">
+      <c r="R92" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-28 08:42:25)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R92"/>
+  <dimension ref="A1:R89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7335,7 +7335,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">9945 </t>
+          <t xml:space="preserve">10007 </t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -7345,12 +7345,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>LACROZE, FEDERICO AV. 1938</t>
+          <t>CABEZON, JOSE LEON 3614</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7388,24 +7388,24 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>-58.440759</v>
+        <v>-58.515037</v>
       </c>
       <c r="N82" t="n">
-        <v>-34.565819</v>
+        <v>-34.589042</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>BLO-L</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7417,22 +7417,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">10007 </t>
+          <t xml:space="preserve">8734 </t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CABEZON, JOSE LEON 3614</t>
+          <t>ARISMENDI 2916</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -7470,10 +7470,10 @@
         <v>1</v>
       </c>
       <c r="M83" t="n">
-        <v>-58.515037</v>
+        <v>-58.479126</v>
       </c>
       <c r="N83" t="n">
-        <v>-34.589042</v>
+        <v>-34.586673</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -7487,7 +7487,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -7499,7 +7499,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">8726 </t>
+          <t xml:space="preserve">10037 </t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -7509,12 +7509,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>HERNANDARIAS 1957</t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -7545,31 +7545,31 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L84" t="n">
         <v>1</v>
       </c>
       <c r="M84" t="n">
-        <v>-58.366665</v>
+        <v>-58.50158</v>
       </c>
       <c r="N84" t="n">
-        <v>-34.646956</v>
+        <v>-34.648954</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>CON-E</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -7581,7 +7581,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">8734 </t>
+          <t xml:space="preserve">10058 </t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7591,12 +7591,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ARISMENDI 2916</t>
+          <t xml:space="preserve">OLIDEN 1187 </t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -7612,12 +7612,12 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -7634,14 +7634,14 @@
         <v>1</v>
       </c>
       <c r="M85" t="n">
-        <v>-58.479126</v>
+        <v>-58.507509</v>
       </c>
       <c r="N85" t="n">
-        <v>-34.586673</v>
+        <v>-34.650225</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
@@ -7651,7 +7651,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7663,7 +7663,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">10037 </t>
+          <t xml:space="preserve">10073 </t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7673,12 +7673,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>GUALEGUAYCHU 3464</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -7694,12 +7694,12 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -7709,17 +7709,17 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L86" t="n">
         <v>1</v>
       </c>
       <c r="M86" t="n">
-        <v>-58.50158</v>
+        <v>-58.511499</v>
       </c>
       <c r="N86" t="n">
-        <v>-34.648954</v>
+        <v>-34.603949</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -7733,7 +7733,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>DEV-C</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -7745,7 +7745,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">10058 </t>
+          <t xml:space="preserve">10151 </t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7755,7 +7755,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">OLIDEN 1187 </t>
+          <t>LAGUNA 1562</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7791,17 +7791,17 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L87" t="n">
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>-58.507509</v>
+        <v>-58.467824</v>
       </c>
       <c r="N87" t="n">
-        <v>-34.650225</v>
+        <v>-34.649072</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -7815,7 +7815,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>PAV-I</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -7827,22 +7827,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">10073 </t>
+          <t>-4992</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU 3464</t>
+          <t>BEYROUTH 4992</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -7858,12 +7858,12 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>REALIZAR CAMBIO DE POSTE POR COLUMNA</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -7877,13 +7877,13 @@
         </is>
       </c>
       <c r="L88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M88" t="n">
-        <v>-58.511499</v>
+        <v>-58.502223</v>
       </c>
       <c r="N88" t="n">
-        <v>-34.603949</v>
+        <v>-34.626887</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -7897,7 +7897,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>DEV-C</t>
+          <t>DEV-H</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -7909,22 +7909,22 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">10097 </t>
+          <t>-4926</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>DESCALZI, NICOLAS 5404</t>
+          <t>BEYROUTH 4926</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -7940,12 +7940,12 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>DESMONTAR COLUMNA</t>
+          <t>CAMBIAR POSTE POR COLUMNA</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -7962,273 +7962,27 @@
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-58.463809</v>
+        <v>-58.501459</v>
       </c>
       <c r="N89" t="n">
-        <v>-34.68275</v>
+        <v>-34.626196</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>DEV-H</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10151 </t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>LAGUNA 1562</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>COLUMNA INCLINADA</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>Aplomo</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="L90" t="n">
-        <v>1</v>
-      </c>
-      <c r="M90" t="n">
-        <v>-58.467824</v>
-      </c>
-      <c r="N90" t="n">
-        <v>-34.649072</v>
-      </c>
-      <c r="O90" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P90" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q90" t="inlineStr">
-        <is>
-          <t>PPT-N</t>
-        </is>
-      </c>
-      <c r="R90" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>-4992</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>5/26/2026</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>BEYROUTH 4992</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>REALIZAR CAMBIO DE POSTE POR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L91" t="n">
-        <v>0</v>
-      </c>
-      <c r="M91" t="n">
-        <v>-58.502223</v>
-      </c>
-      <c r="N91" t="n">
-        <v>-34.626887</v>
-      </c>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P91" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>DEV-H</t>
-        </is>
-      </c>
-      <c r="R91" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>-4926</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>5/26/2026</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>BEYROUTH 4926</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L92" t="n">
-        <v>1</v>
-      </c>
-      <c r="M92" t="n">
-        <v>-58.501459</v>
-      </c>
-      <c r="N92" t="n">
-        <v>-34.626196</v>
-      </c>
-      <c r="O92" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P92" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q92" t="inlineStr">
-        <is>
-          <t>DEV-H</t>
-        </is>
-      </c>
-      <c r="R92" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 11:48:06)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -4063,7 +4063,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107575</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107549</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107595</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107070</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814107603</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -6539,7 +6539,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>814108508</t>
+        </is>
+      </c>
       <c r="H72" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -7359,7 +7363,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>814108006</t>
+        </is>
+      </c>
       <c r="H82" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -7441,7 +7449,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>814108096</t>
+        </is>
+      </c>
       <c r="H83" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -7769,10 +7781,14 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>814107868</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>REALIZAR CAMBIO DE POSTE POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -7787,7 +7803,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L87" t="n">
@@ -7851,10 +7867,14 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>814107901</t>
+        </is>
+      </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -7869,7 +7889,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L88" t="n">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 13:06:04)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -6707,7 +6707,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>814109429</t>
+        </is>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -6789,7 +6793,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>814109781</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>
@@ -7281,7 +7289,11 @@
           <t>INGEME</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>814109840</t>
+        </is>
+      </c>
       <c r="H81" t="inlineStr">
         <is>
           <t>CAMBIAR COLUMNA</t>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-02 15:37:49)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R88"/>
+  <dimension ref="A1:R99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,17 +439,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>801645368</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>801645368</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -617,17 +617,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>801901755</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>801901755</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -703,17 +703,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>802657454</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>802657454</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -789,17 +789,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>802843289</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>802843289</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -875,17 +875,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>803983204</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>803983204</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>806945058</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>806945058</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1047,17 +1047,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808579768</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>808579768</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1133,17 +1133,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>808918698</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>808918698</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>809007047</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>809007047</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1305,17 +1305,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810056868</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>810056868</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1391,17 +1391,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>ICD31468700</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>ICD31468700</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1477,17 +1477,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810132548</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>810132548</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1563,17 +1563,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810244452</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>810244452</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1649,17 +1649,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810259143</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>810259143</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1735,17 +1735,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810333010</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>810333010</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1821,17 +1821,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810404280</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>810404280</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1907,17 +1907,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810416660</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>810416660</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1993,17 +1993,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2079,17 +2079,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2165,17 +2165,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>810651269</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2251,17 +2251,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2337,17 +2337,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810820624</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>810820624</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2423,17 +2423,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>810820533</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>810820533</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2509,17 +2509,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811131640</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>811131640</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2595,17 +2595,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198627</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>811198627</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811181316</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>811181316</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2767,17 +2767,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811198686</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>811198686</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2853,17 +2853,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2935,17 +2935,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811299433</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>811299433</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3021,17 +3021,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454117</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>811454117</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3107,17 +3107,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811454109</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>811454109</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3193,17 +3193,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811453943</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>811453943</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3279,17 +3279,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626897</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>811626897</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3365,17 +3365,17 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3451,17 +3451,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627070</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>811627070</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3537,17 +3537,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>811627041</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>811627041</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3623,17 +3623,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440197</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>812440197</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3709,17 +3709,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812440520</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>812440520</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3795,17 +3795,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812503637</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>812503637</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3881,17 +3881,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812503649</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>812503649</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3967,17 +3967,17 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812503647</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>812503647</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4053,17 +4053,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107575</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>814107575</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4139,17 +4139,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107549</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>814107549</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4225,17 +4225,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107595</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>814107595</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4311,17 +4311,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107070</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>814107070</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4397,17 +4397,17 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107603</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>814107603</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4483,17 +4483,17 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879612</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>812879612</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4565,17 +4565,17 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879773</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>812879773</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4651,17 +4651,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879780</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>812879780</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4737,17 +4737,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812879976</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>812879976</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4823,17 +4823,17 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880445</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>812880445</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4909,17 +4909,17 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>812880729</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>812880729</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4991,17 +4991,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046368</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>813046368</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -5077,17 +5077,17 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046780</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>813046780</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5163,17 +5163,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046813</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>813046813</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5249,17 +5249,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046868</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>813046868</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -5331,17 +5331,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813046870</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>813046870</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5417,17 +5417,17 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047531</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>813047531</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -5503,17 +5503,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813047700</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>813047700</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5589,17 +5589,17 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304416</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>813304416</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5675,17 +5675,17 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304660</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>813304660</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -5761,17 +5761,17 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304738</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>813304738</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5847,17 +5847,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813304912</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>813304912</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5933,17 +5933,17 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813350688</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>813350688</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -6019,17 +6019,17 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813352594</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>813352594</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -6105,17 +6105,17 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813353208</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>813353208</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -6191,17 +6191,17 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631418</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>813631418</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -6277,17 +6277,17 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631419</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>813631419</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -6359,17 +6359,17 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631455</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>813631455</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -6445,17 +6445,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>813631875</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>813631875</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -6531,17 +6531,17 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108508</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>814108508</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6615,17 +6615,17 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
           <t xml:space="preserve">DESMONTAR POSTE MADERA </t>
@@ -6699,17 +6699,17 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109429</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>814109429</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6785,17 +6785,17 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109781</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>814109781</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -6871,15 +6871,19 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111103</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -6887,7 +6891,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -6953,15 +6957,19 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111112</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -6969,7 +6977,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -7035,15 +7043,19 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111113</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -7051,7 +7063,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -7117,15 +7129,19 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111159</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
           <t>COLUMN INCLINADA</t>
@@ -7133,7 +7149,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -7199,15 +7215,19 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111168</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H80" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -7215,7 +7235,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -7281,17 +7301,17 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814109840</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>814109840</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -7367,17 +7387,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108006</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>814108006</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -7453,17 +7473,17 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814108096</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>814108096</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -7539,15 +7559,19 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111720</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H84" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -7555,7 +7579,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -7621,15 +7645,19 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111762</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H85" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -7637,7 +7665,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -7703,15 +7731,19 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814111819</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
       <c r="H86" t="inlineStr">
         <is>
           <t>COLUMNA INCLINADA</t>
@@ -7719,7 +7751,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -7785,17 +7817,17 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107868</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>814107868</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -7871,17 +7903,17 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>814107901</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>814107901</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -7931,6 +7963,952 @@
       <c r="R88" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>-784</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>PERON, EVA AV. 7255</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>814125579</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L89" t="n">
+        <v>1</v>
+      </c>
+      <c r="M89" t="n">
+        <v>-58.499701</v>
+      </c>
+      <c r="N89" t="n">
+        <v>-34.672846</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>PAV-K</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>-793</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>BOGOTA 4046</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>814125611</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L90" t="n">
+        <v>1</v>
+      </c>
+      <c r="M90" t="n">
+        <v>-58.484954</v>
+      </c>
+      <c r="N90" t="n">
+        <v>-34.631036</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>DEV-L</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2DEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>-794</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>BOGOTA 4090</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>814125613</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L91" t="n">
+        <v>1</v>
+      </c>
+      <c r="M91" t="n">
+        <v>-58.485508</v>
+      </c>
+      <c r="N91" t="n">
+        <v>-34.631175</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>DEV-L</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2DEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>-795</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CABEZON, JOSE LEON 3494</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>814125617</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>base podrida</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
+        <v>1</v>
+      </c>
+      <c r="M92" t="n">
+        <v>-58.51297</v>
+      </c>
+      <c r="N92" t="n">
+        <v>-34.587773</v>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>PUE-J</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>-806</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>MEDINA 422</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>814125658</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L93" t="n">
+        <v>1</v>
+      </c>
+      <c r="M93" t="n">
+        <v>-58.48802</v>
+      </c>
+      <c r="N93" t="n">
+        <v>-34.641075</v>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>PCH-S</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2PCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>-807</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>MEDINA 427</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>814125659</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L94" t="n">
+        <v>1</v>
+      </c>
+      <c r="M94" t="n">
+        <v>-58.488051</v>
+      </c>
+      <c r="N94" t="n">
+        <v>-34.641152</v>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>PCH-S</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2PCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>-811</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>MORETO 1635</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>814125668</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>base corroida</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L95" t="n">
+        <v>1</v>
+      </c>
+      <c r="M95" t="n">
+        <v>-58.477118</v>
+      </c>
+      <c r="N95" t="n">
+        <v>-34.652322</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>PAV-O</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>-812</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>MURATURE 4536</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>1</v>
+      </c>
+      <c r="M96" t="n">
+        <v>-58.496245</v>
+      </c>
+      <c r="N96" t="n">
+        <v>-34.625987</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>DEV-I</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>-817</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>CISNEROS, VIRREY 1699</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>814125680</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>podrida en base</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L97" t="n">
+        <v>1</v>
+      </c>
+      <c r="M97" t="n">
+        <v>-58.470179</v>
+      </c>
+      <c r="N97" t="n">
+        <v>-34.611301</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>NRA-K</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>PIZARRO 7485</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>814125705</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
+        <v>1</v>
+      </c>
+      <c r="M98" t="n">
+        <v>-58.518126</v>
+      </c>
+      <c r="N98" t="n">
+        <v>-34.658739</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>PAV-I</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>-822</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>6/2/2026</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>RODO, JOSE E. 4011</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>814125706</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>inclinada</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L99" t="n">
+        <v>1</v>
+      </c>
+      <c r="M99" t="n">
+        <v>-58.481618</v>
+      </c>
+      <c r="N99" t="n">
+        <v>-34.640762</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>PCH-P</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-10 15:53:11)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R80"/>
+  <dimension ref="A1:R78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3345,17 +3345,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>900009605910</t>
+          <t>8480</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>3/6/2026</t>
+          <t>3/5/2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">BORDABEHERE ENZO 2801 </t>
+          <t>NAZCA AV. 3312</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>814107549</t>
+          <t>814107595</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3395,17 +3395,17 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.480297</v>
+        <v>-58.492236</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.600118</v>
+        <v>-34.598228</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>PUE-A</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3431,22 +3431,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>8480</t>
+          <t>8554</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>3/5/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>NAZCA AV. 3312</t>
+          <t>OLIDEN 55</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>814107595</t>
+          <t>814107070</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3481,21 +3481,21 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.492236</v>
+        <v>-58.517269</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.598228</v>
+        <v>-34.639879</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>PAV-B</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3517,22 +3517,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>8554</t>
+          <t>-771</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>2/18/2026</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>OLIDEN 55</t>
+          <t>SAN BLAS 4112</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>814107070</t>
+          <t>814107603</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3567,17 +3567,17 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.517269</v>
+        <v>-58.494458</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.639879</v>
+        <v>-34.620078</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PAV-B</t>
+          <t>DEV-J</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3603,22 +3603,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>-771</t>
+          <t xml:space="preserve">8618 </t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2/18/2026</t>
+          <t>3/17/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SAN BLAS 4112</t>
+          <t>VALLEJOS 4319</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>814107603</t>
+          <t>812879612</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE Y COLOCAR COLUMNA</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3651,23 +3651,19 @@
           <t>Sin equipos</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Poste</t>
-        </is>
-      </c>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.494458</v>
+        <v>-58.51875</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.620078</v>
+        <v>-34.598858</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3677,7 +3673,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>DEV-J</t>
+          <t>PUE-P</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3689,22 +3685,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">8618 </t>
+          <t>8882</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>3/17/2026</t>
+          <t>3/18/2026</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>VALLEJOS 4319</t>
+          <t>EL PROFETA DE LA PAMPA 4523</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3714,7 +3710,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>812879612</t>
+          <t>812879773</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3724,7 +3720,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y COLOCAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3734,22 +3730,26 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.51875</v>
+        <v>-58.477211</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.598858</v>
+        <v>-34.652708</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>PUE-P</t>
+          <t>PAV-O</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3771,17 +3771,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>8882</t>
+          <t>00239146</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>3/18/2026</t>
+          <t>3/19/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>EL PROFETA DE LA PAMPA 4523</t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>812879773</t>
+          <t>812879780</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3816,22 +3816,22 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L40" t="n">
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.477211</v>
+        <v>-58.50158</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.652708</v>
+        <v>-34.648954</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>PAV-O</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3857,22 +3857,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>00239146</t>
+          <t xml:space="preserve">7460 </t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>3/19/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>TERRADA 2720</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>812879780</t>
+          <t>812879976</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3892,12 +3892,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>RIENDA A PIQUE CORTADA</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -3911,17 +3911,17 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.50158</v>
+        <v>-58.486103</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.648954</v>
+        <v>-34.603895</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>NRA-P</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3943,7 +3943,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">7460 </t>
+          <t>00000609</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3953,12 +3953,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>TERRADA 2720</t>
+          <t>ZELADA 4402</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>812879976</t>
+          <t>812880445</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3978,12 +3978,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>RIENDA A PIQUE CORTADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3993,21 +3993,21 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.486103</v>
+        <v>-58.48834</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.603895</v>
+        <v>-34.641018</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -4017,34 +4017,30 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>00000609</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>3/21/2026</t>
-        </is>
-      </c>
+          <t xml:space="preserve">900009880510 </t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ZELADA 4402</t>
+          <t>GUTENBERG 4150</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4054,7 +4050,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>812880445</t>
+          <t>813046368</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4064,7 +4060,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR POSTE POR COLUMNA</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4086,14 +4082,14 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.48834</v>
+        <v>-58.516791</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.641018</v>
+        <v>-34.596662</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -4103,30 +4099,34 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PUE-P</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009880510 </t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
+          <t>S00373014</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>4/11/2026</t>
+        </is>
+      </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GUTENBERG 4150</t>
+          <t>BYRON 150</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>813046368</t>
+          <t>813046780</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4168,14 +4168,14 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.516791</v>
+        <v>-58.501659</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.596662</v>
+        <v>-34.63959</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>PUE-P</t>
+          <t>PAV-F</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4197,7 +4197,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S00373014</t>
+          <t>8831</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BYRON 150</t>
+          <t>FLORES VENACIO GRAL 4567</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4222,7 +4222,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>813046780</t>
+          <t>813046868</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4253,25 +4253,21 @@
       <c r="L45" t="n">
         <v>1</v>
       </c>
-      <c r="M45" t="n">
-        <v>-58.501659</v>
-      </c>
-      <c r="N45" t="n">
-        <v>-34.63959</v>
-      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>No clasificado, consultar con mantenimiento</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>PAV-F</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4283,7 +4279,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>8831</t>
+          <t>8832</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4293,7 +4289,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>FLORES VENACIO GRAL 4567</t>
+          <t>SANTO TOME 6674</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -4308,7 +4304,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>813046868</t>
+          <t>813046870</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4339,21 +4335,25 @@
       <c r="L46" t="n">
         <v>1</v>
       </c>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>-58.528021</v>
+      </c>
+      <c r="N46" t="n">
+        <v>-34.627813</v>
+      </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>No clasificado, consultar con mantenimiento</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>DEV-O</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4365,7 +4365,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>8832</t>
+          <t>8686</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4375,7 +4375,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SANTO TOME 6674</t>
+          <t>CERVANTES 650</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>813046870</t>
+          <t>813047531</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4422,10 +4422,10 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>-58.528021</v>
+        <v>-58.497176</v>
       </c>
       <c r="N47" t="n">
-        <v>-34.627813</v>
+        <v>-34.631131</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -4439,19 +4439,19 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>DEV-O</t>
+          <t>DEV-M</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>8686</t>
+          <t>S00391032</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -4461,12 +4461,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CERVANTES 650</t>
+          <t>MARISCAL SOLANO LOPEZ 3312</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>813047531</t>
+          <t>813047700</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE Y COLOCAR COLUMNA</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4508,14 +4508,14 @@
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>-58.497176</v>
+        <v>-58.501067</v>
       </c>
       <c r="N48" t="n">
-        <v>-34.631131</v>
+        <v>-34.596916</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -4525,29 +4525,29 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>DEV-M</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S00391032</t>
+          <t>S00400580</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/14/2026</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MARISCAL SOLANO LOPEZ 3312</t>
+          <t>BORDABEHERE, ENZO 2802</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>813047700</t>
+          <t>813304660</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE Y COLOCAR COLUMNA</t>
+          <t>CAMBIAR POSTE DE MADERA POR COLUMNA</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4594,10 +4594,10 @@
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>-58.501067</v>
+        <v>-58.480405</v>
       </c>
       <c r="N49" t="n">
-        <v>-34.596916</v>
+        <v>-34.600087</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>PUE-A</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4623,22 +4623,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S00400580</t>
+          <t>8954</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>4/14/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BORDABEHERE, ENZO 2802</t>
+          <t>FLORES, VENANCIO, GRAL. 4550</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>813304660</t>
+          <t>813350688</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE DE MADERA POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4680,14 +4680,14 @@
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-58.480405</v>
+        <v>-58.490636</v>
       </c>
       <c r="N50" t="n">
-        <v>-34.600087</v>
+        <v>-34.634459</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -4697,34 +4697,34 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>PUE-A</t>
+          <t>DEV-M</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>8954</t>
+          <t>9022</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>4/21/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 4550</t>
+          <t xml:space="preserve">MAGARIÑOS CERVANTES, A. 2072 </t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4734,7 +4734,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>813350688</t>
+          <t>813352594</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4766,14 +4766,14 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>-58.490636</v>
+        <v>-58.46936</v>
       </c>
       <c r="N51" t="n">
-        <v>-34.634459</v>
+        <v>-34.60805</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -4783,19 +4783,19 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>DEV-M</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>9022</t>
+          <t>S00463265</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4805,12 +4805,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGARIÑOS CERVANTES, A. 2072 </t>
+          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>813352594</t>
+          <t>813353208</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -4852,14 +4852,14 @@
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>-58.46936</v>
+        <v>-58.508425</v>
       </c>
       <c r="N52" t="n">
-        <v>-34.60805</v>
+        <v>-34.653353</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4881,22 +4881,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S00463265</t>
+          <t>S00369718</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
+          <t>FLORES, VENANCIO, GRAL. 4568</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>813353208</t>
+          <t>813631875</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4938,10 +4938,10 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>-58.508425</v>
+        <v>-58.490942</v>
       </c>
       <c r="N53" t="n">
-        <v>-34.653353</v>
+        <v>-34.634502</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -4955,34 +4955,34 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>DEV-M</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S00488557</t>
+          <t xml:space="preserve">9139 </t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>COSQUIN 296</t>
+          <t>MOSCONI GENERAL AV. 3327</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>813631455</t>
+          <t>814108508</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -5024,14 +5024,14 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>-58.523272</v>
+        <v>-58.508028</v>
       </c>
       <c r="N54" t="n">
-        <v>-34.642619</v>
+        <v>-34.589722</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PAV-C</t>
+          <t>PUE-N</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5053,22 +5053,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S00369718</t>
+          <t>S00497584</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>FLORES, VENANCIO, GRAL. 4568</t>
+          <t>SOLANO LOPEZ, F., MARISCAL 3280</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5076,11 +5076,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>813631875</t>
-        </is>
-      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -5088,12 +5084,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t xml:space="preserve">DESMONTAR POSTE MADERA </t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -5110,14 +5106,14 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>-58.490942</v>
+        <v>-58.500541</v>
       </c>
       <c r="N55" t="n">
-        <v>-34.634502</v>
+        <v>-34.596596</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -5127,19 +5123,19 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>DEV-M</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">9139 </t>
+          <t xml:space="preserve">900009976210 </t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5149,7 +5145,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>MOSCONI GENERAL AV. 3327</t>
+          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5164,7 +5160,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>814108508</t>
+          <t>814109781</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -5196,10 +5192,10 @@
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>-58.508028</v>
+        <v>-58.477456</v>
       </c>
       <c r="N56" t="n">
-        <v>-34.589722</v>
+        <v>-34.614971</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -5213,7 +5209,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PUE-N</t>
+          <t>NRA-M</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5225,7 +5221,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S00497584</t>
+          <t>9938</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -5235,7 +5231,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SOLANO LOPEZ, F., MARISCAL 3280</t>
+          <t>QUESADA 5060</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -5248,7 +5244,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>814111103</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -5256,12 +5256,12 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t xml:space="preserve">DESMONTAR POSTE MADERA </t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -5278,10 +5278,10 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>-58.500541</v>
+        <v>-58.489366</v>
       </c>
       <c r="N57" t="n">
-        <v>-34.596596</v>
+        <v>-34.568013</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5295,7 +5295,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5307,7 +5307,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009976210 </t>
+          <t xml:space="preserve">9940 </t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
+          <t>QUESADA 5210</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>814109781</t>
+          <t>814111113</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5364,10 +5364,10 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>-58.477456</v>
+        <v>-58.491219</v>
       </c>
       <c r="N58" t="n">
-        <v>-34.614971</v>
+        <v>-34.568967</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>NRA-M</t>
+          <t>PUE-F</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5393,7 +5393,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>9938</t>
+          <t xml:space="preserve">9942 </t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>QUESADA 5060</t>
+          <t>CAPDEVILA 3057</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>814111103</t>
+          <t>814111159</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -5428,7 +5428,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>COLUMN INCLINADA</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5450,10 +5450,10 @@
         <v>1</v>
       </c>
       <c r="M59" t="n">
-        <v>-58.489366</v>
+        <v>-58.490684</v>
       </c>
       <c r="N59" t="n">
-        <v>-34.568013</v>
+        <v>-34.569213</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -5479,7 +5479,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">9940 </t>
+          <t xml:space="preserve">10007 </t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>QUESADA 5210</t>
+          <t>CABEZON, JOSE LEON 3614</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5504,7 +5504,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>814111113</t>
+          <t>814109840</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5536,10 +5536,10 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>-58.491219</v>
+        <v>-58.515037</v>
       </c>
       <c r="N60" t="n">
-        <v>-34.568967</v>
+        <v>-34.589042</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5565,22 +5565,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">9942 </t>
+          <t xml:space="preserve">8734 </t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CAPDEVILA 3057</t>
+          <t>ARISMENDI 2916</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>814111159</t>
+          <t>814108006</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>COLUMN INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5622,10 +5622,10 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>-58.490684</v>
+        <v>-58.479126</v>
       </c>
       <c r="N61" t="n">
-        <v>-34.569213</v>
+        <v>-34.586673</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -5639,7 +5639,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PUE-F</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5651,22 +5651,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">10007 </t>
+          <t xml:space="preserve">10037 </t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CABEZON, JOSE LEON 3614</t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5676,7 +5676,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>814109840</t>
+          <t>814108096</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -5701,21 +5701,21 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L62" t="n">
         <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>-58.515037</v>
+        <v>-58.50158</v>
       </c>
       <c r="N62" t="n">
-        <v>-34.589042</v>
+        <v>-34.648954</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -5725,7 +5725,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5737,7 +5737,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">8734 </t>
+          <t xml:space="preserve">10058 </t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5747,12 +5747,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ARISMENDI 2916</t>
+          <t xml:space="preserve">OLIDEN 1187 </t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5762,7 +5762,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>814108006</t>
+          <t>814111720</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5794,14 +5794,14 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>-58.479126</v>
+        <v>-58.507509</v>
       </c>
       <c r="N63" t="n">
-        <v>-34.586673</v>
+        <v>-34.650225</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5823,7 +5823,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">10037 </t>
+          <t xml:space="preserve">10073 </t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5833,12 +5833,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>GUALEGUAYCHU 3464</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5848,7 +5848,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>814108096</t>
+          <t>814111762</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -5873,17 +5873,17 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L64" t="n">
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>-58.50158</v>
+        <v>-58.511499</v>
       </c>
       <c r="N64" t="n">
-        <v>-34.648954</v>
+        <v>-34.603949</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>DEV-C</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -5909,7 +5909,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">10058 </t>
+          <t xml:space="preserve">10151 </t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">OLIDEN 1187 </t>
+          <t>LAGUNA 1562</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -5934,7 +5934,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>814111720</t>
+          <t>814111819</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -5959,17 +5959,17 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L65" t="n">
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>-58.507509</v>
+        <v>-58.467824</v>
       </c>
       <c r="N65" t="n">
-        <v>-34.650225</v>
+        <v>-34.649072</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>PAV-I</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -5995,22 +5995,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">10073 </t>
+          <t>-4992</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU 3464</t>
+          <t>BEYROUTH 4992</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>814111762</t>
+          <t>814107868</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -6030,7 +6030,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6045,17 +6045,17 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M66" t="n">
-        <v>-58.511499</v>
+        <v>-58.502223</v>
       </c>
       <c r="N66" t="n">
-        <v>-34.603949</v>
+        <v>-34.626887</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -6069,7 +6069,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>DEV-C</t>
+          <t>DEV-H</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6081,22 +6081,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">10151 </t>
+          <t>-4926</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>5/26/2026</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LAGUNA 1562</t>
+          <t>BEYROUTH 4926</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>814111819</t>
+          <t>814107901</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -6116,7 +6116,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6131,17 +6131,17 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L67" t="n">
         <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>-58.467824</v>
+        <v>-58.501459</v>
       </c>
       <c r="N67" t="n">
-        <v>-34.649072</v>
+        <v>-34.626196</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -6155,7 +6155,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>DEV-H</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6167,22 +6167,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>-4992</t>
+          <t>-784</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>BEYROUTH 4992</t>
+          <t>PERON, EVA AV. 7255</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>814107868</t>
+          <t>814125579</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -6202,7 +6202,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6217,17 +6217,17 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>-58.502223</v>
+        <v>-58.499701</v>
       </c>
       <c r="N68" t="n">
-        <v>-34.626887</v>
+        <v>-34.672846</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -6241,7 +6241,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>DEV-H</t>
+          <t>PAV-K</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6253,17 +6253,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>-4926</t>
+          <t>-793</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>5/26/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>BEYROUTH 4926</t>
+          <t>BOGOTA 4046</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>814107901</t>
+          <t>814125611</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6303,17 +6303,17 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L69" t="n">
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>-58.501459</v>
+        <v>-58.484954</v>
       </c>
       <c r="N69" t="n">
-        <v>-34.626196</v>
+        <v>-34.631036</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -6327,19 +6327,19 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>DEV-H</t>
+          <t>DEV-L</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>-784</t>
+          <t>-794</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -6349,12 +6349,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PERON, EVA AV. 7255</t>
+          <t>BOGOTA 4090</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>814125579</t>
+          <t>814125613</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -6396,10 +6396,10 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>-58.499701</v>
+        <v>-58.485508</v>
       </c>
       <c r="N70" t="n">
-        <v>-34.672846</v>
+        <v>-34.631175</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -6413,19 +6413,19 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>PAV-K</t>
+          <t>DEV-L</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>-793</t>
+          <t>-795</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -6435,12 +6435,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>BOGOTA 4046</t>
+          <t>CABEZON, JOSE LEON 3494</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -6450,7 +6450,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>814125611</t>
+          <t>814125617</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base podrida</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6482,14 +6482,14 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>-58.484954</v>
+        <v>-58.51297</v>
       </c>
       <c r="N71" t="n">
-        <v>-34.631036</v>
+        <v>-34.587773</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -6499,19 +6499,19 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>-794</t>
+          <t>-806</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6521,7 +6521,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>BOGOTA 4090</t>
+          <t>MEDINA 422</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>814125613</t>
+          <t>814125658</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -6561,17 +6561,17 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L72" t="n">
         <v>1</v>
       </c>
       <c r="M72" t="n">
-        <v>-58.485508</v>
+        <v>-58.48802</v>
       </c>
       <c r="N72" t="n">
-        <v>-34.631175</v>
+        <v>-34.641075</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -6585,19 +6585,19 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>-795</t>
+          <t>-807</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6607,12 +6607,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CABEZON, JOSE LEON 3494</t>
+          <t>MEDINA 427</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6622,7 +6622,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>814125617</t>
+          <t>814125659</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>base podrida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -6654,14 +6654,14 @@
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>-58.51297</v>
+        <v>-58.488051</v>
       </c>
       <c r="N73" t="n">
-        <v>-34.587773</v>
+        <v>-34.641152</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -6671,19 +6671,19 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>-806</t>
+          <t>-811</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6693,12 +6693,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MEDINA 422</t>
+          <t>MORETO 1635</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>814125658</t>
+          <t>814125668</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -6733,17 +6733,17 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L74" t="n">
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>-58.48802</v>
+        <v>-58.477118</v>
       </c>
       <c r="N74" t="n">
-        <v>-34.641075</v>
+        <v>-34.652322</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -6757,19 +6757,19 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>PAV-O</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>-807</t>
+          <t>-812</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -6779,7 +6779,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>MEDINA 427</t>
+          <t>MURATURE 4536</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -6794,7 +6794,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>814125659</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -6826,10 +6826,10 @@
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>-58.488051</v>
+        <v>-58.496245</v>
       </c>
       <c r="N75" t="n">
-        <v>-34.641152</v>
+        <v>-34.625987</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6843,19 +6843,19 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>DEV-I</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>-811</t>
+          <t>-817</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -6865,12 +6865,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>MORETO 1635</t>
+          <t>CISNEROS, VIRREY 1699</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>814125668</t>
+          <t>814125680</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -6890,7 +6890,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>podrida en base</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -6912,14 +6912,14 @@
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>-58.477118</v>
+        <v>-58.470179</v>
       </c>
       <c r="N76" t="n">
-        <v>-34.652322</v>
+        <v>-34.611301</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
@@ -6929,7 +6929,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PAV-O</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6941,7 +6941,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>-812</t>
+          <t>-821</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -6951,12 +6951,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>MURATURE 4536</t>
+          <t>PIZARRO 7485</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125705</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -6986,7 +6986,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -6998,10 +6998,10 @@
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-58.496245</v>
+        <v>-58.518126</v>
       </c>
       <c r="N77" t="n">
-        <v>-34.625987</v>
+        <v>-34.658739</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>DEV-I</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7027,7 +7027,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>-817</t>
+          <t>-822</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -7037,12 +7037,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CISNEROS, VIRREY 1699</t>
+          <t>RODO, JOSE E. 4011</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7052,7 +7052,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>814125680</t>
+          <t>814125706</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -7062,7 +7062,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>podrida en base</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -7084,14 +7084,14 @@
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>-58.470179</v>
+        <v>-58.481618</v>
       </c>
       <c r="N78" t="n">
-        <v>-34.611301</v>
+        <v>-34.640762</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -7101,182 +7101,10 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>PCH-P</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>-821</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>PIZARRO 7485</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>814125705</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L79" t="n">
-        <v>1</v>
-      </c>
-      <c r="M79" t="n">
-        <v>-58.518126</v>
-      </c>
-      <c r="N79" t="n">
-        <v>-34.658739</v>
-      </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P79" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q79" t="inlineStr">
-        <is>
-          <t>PAV-I</t>
-        </is>
-      </c>
-      <c r="R79" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>-822</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>RODO, JOSE E. 4011</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>814125706</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L80" t="n">
-        <v>1</v>
-      </c>
-      <c r="M80" t="n">
-        <v>-58.481618</v>
-      </c>
-      <c r="N80" t="n">
-        <v>-34.640762</v>
-      </c>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q80" t="inlineStr">
-        <is>
-          <t>PCH-P</t>
-        </is>
-      </c>
-      <c r="R80" t="inlineStr">
         <is>
           <t>ARATO-25058.PO.2PCH</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-19 14:54:18)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R47"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4033,7 +4033,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>-811</t>
+          <t>-812</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4043,12 +4043,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MORETO 1635</t>
+          <t>MURATURE 4536</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>814125668</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -4090,10 +4090,10 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>-58.477118</v>
+        <v>-58.496245</v>
       </c>
       <c r="N43" t="n">
-        <v>-34.652322</v>
+        <v>-34.625987</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>PAV-O</t>
+          <t>DEV-I</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4119,7 +4119,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>-812</t>
+          <t>-817</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4129,12 +4129,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MURATURE 4536</t>
+          <t>CISNEROS, VIRREY 1699</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125680</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>podrida en base</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -4176,14 +4176,14 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>-58.496245</v>
+        <v>-58.470179</v>
       </c>
       <c r="N44" t="n">
-        <v>-34.625987</v>
+        <v>-34.611301</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -4193,7 +4193,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>DEV-I</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4205,7 +4205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>-817</t>
+          <t>-821</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4215,12 +4215,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CISNEROS, VIRREY 1699</t>
+          <t>PIZARRO 7485</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>814125680</t>
+          <t>814125705</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>podrida en base</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4262,14 +4262,14 @@
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>-58.470179</v>
+        <v>-58.518126</v>
       </c>
       <c r="N45" t="n">
-        <v>-34.611301</v>
+        <v>-34.658739</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -4279,184 +4279,12 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>-821</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>PIZARRO 7485</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>814125705</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L46" t="n">
-        <v>1</v>
-      </c>
-      <c r="M46" t="n">
-        <v>-58.518126</v>
-      </c>
-      <c r="N46" t="n">
-        <v>-34.658739</v>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>PAV-I</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>-822</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>RODO, JOSE E. 4011</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>814125706</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L47" t="n">
-        <v>1</v>
-      </c>
-      <c r="M47" t="n">
-        <v>-58.481618</v>
-      </c>
-      <c r="N47" t="n">
-        <v>-34.640762</v>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>PCH-P</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-24 13:16:05)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:R38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1371,17 +1371,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>-646</t>
+          <t>8482</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10/20/2025</t>
+          <t>10/21/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Andres Lamas 1845</t>
+          <t>San Blas 2591</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>810404280</t>
+          <t>810416660</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1428,10 +1428,10 @@
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>-58.468222</v>
+        <v>-58.477427</v>
       </c>
       <c r="N12" t="n">
-        <v>-34.608355</v>
+        <v>-34.609261</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1457,22 +1457,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8482</t>
+          <t>7622</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10/21/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>San Blas 2591</t>
+          <t>MIRALLA 950</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>810416660</t>
+          <t>01233440</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1514,14 +1514,14 @@
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>-58.477427</v>
+        <v>-58.50161</v>
       </c>
       <c r="N13" t="n">
-        <v>-34.609261</v>
+        <v>-34.647648</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>PAV-?</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1543,22 +1543,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7622</t>
+          <t>7709</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/30/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MIRALLA 950</t>
+          <t>SAN BLAS 2891</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>01233440</t>
+          <t>810487021</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1600,14 +1600,14 @@
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>-58.50161</v>
+        <v>-58.48121</v>
       </c>
       <c r="N14" t="n">
-        <v>-34.647648</v>
+        <v>-34.61126</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>PAV-?</t>
+          <t>NRA-Q</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1629,32 +1629,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>7709</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10/30/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SAN BLAS 2891</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>810487021</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1686,14 +1686,14 @@
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>-58.48121</v>
+        <v>-58.510994</v>
       </c>
       <c r="N15" t="n">
-        <v>-34.61126</v>
+        <v>-34.655027</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NRA-Q</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1715,17 +1715,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>-670</t>
+          <t>S01112737</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>11/20/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Timoteo Gordillo 1666</t>
+          <t>RODO, JOSE E. 4799</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1735,12 +1735,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pendiente de Traspaso PROPIO</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>810820822</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1772,10 +1772,10 @@
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>-58.510994</v>
+        <v>-58.491325</v>
       </c>
       <c r="N16" t="n">
-        <v>-34.655027</v>
+        <v>-34.647761</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>PAV-H</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1801,7 +1801,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>S01112737</t>
+          <t>7867</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1811,12 +1811,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>RODO, JOSE E. 4799</t>
+          <t>DIAZ, CESAR, GRAL. 1450</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>810820822</t>
+          <t>810820533</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1851,21 +1851,21 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L17" t="n">
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.491325</v>
+        <v>-58.461219</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.647761</v>
+        <v>-34.605928</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>PAV-H</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1887,22 +1887,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>7867</t>
+          <t>-706</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11/20/2025</t>
+          <t>12/17/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DIAZ, CESAR, GRAL. 1450</t>
+          <t>PAZ, MARCOS 1505</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>810820533</t>
+          <t>811181316</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1937,21 +1937,21 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.461219</v>
+        <v>-58.500094</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.605928</v>
+        <v>-34.626115</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>DEV-I</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1973,22 +1973,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>-706</t>
+          <t>7988</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>12/17/2025</t>
+          <t>12/29/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PAZ, MARCOS 1505</t>
+          <t>REMEDIOS 3285</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>811181316</t>
+          <t>811299402</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2023,17 +2023,17 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.500094</v>
+        <v>-58.471183</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.626115</v>
+        <v>-34.638988</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2047,34 +2047,30 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>DEV-I</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
+          <t>PCH-O</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7988</t>
+          <t>7987</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12/29/2025</t>
+          <t>12/30/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>REMEDIOS 3285</t>
+          <t>Terrada 2309</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2084,7 +2080,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>811299402</t>
+          <t>811299433</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2109,21 +2105,21 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.471183</v>
+        <v>-58.482084</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.638988</v>
+        <v>-34.608289</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2133,25 +2129,29 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PCH-O</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr"/>
+          <t>NRA-P</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>7987</t>
+          <t>S01389798</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>12/30/2025</t>
+          <t>1/12/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Terrada 2309</t>
+          <t>GUALEGUAYCHU 4682</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>811299433</t>
+          <t>811453943</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2191,17 +2191,17 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.482084</v>
+        <v>-58.518214</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.608289</v>
+        <v>-34.596516</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>PUE-O</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2227,22 +2227,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S01204059</t>
+          <t>S01447520</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1/12/2026</t>
+          <t>1/29/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BUFANO, ALFREDO R. 2580</t>
+          <t>FALCON, RAMON L.,CNEL. 4326</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>811454109</t>
+          <t>811626894</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2284,14 +2284,14 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.478411</v>
+        <v>-58.487715</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.6039</v>
+        <v>-34.636671</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2301,34 +2301,34 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>PCH-S</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2PCH</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>S01389798</t>
+          <t>S00036520</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1/12/2026</t>
+          <t>2/4/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU 4682</t>
+          <t>SEGUROLA AV. 856</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>811453943</t>
+          <t>811627070</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2370,14 +2370,14 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.518214</v>
+        <v>-58.490765</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.596516</v>
+        <v>-34.627337</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>PUE-O</t>
+          <t>DEV-I</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2399,22 +2399,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>S01447520</t>
+          <t>8481</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1/29/2026</t>
+          <t>2/23/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FALCON, RAMON L.,CNEL. 4326</t>
+          <t>CISNEROS, VIRREY 1610</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>811626894</t>
+          <t>812440520</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2449,21 +2449,21 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L24" t="n">
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.487715</v>
+        <v>-58.469727</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.636671</v>
+        <v>-34.612013</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2473,34 +2473,34 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>PCH-S</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2PCH</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>S00036520</t>
+          <t>8554</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2/4/2026</t>
+          <t>3/9/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SEGUROLA AV. 856</t>
+          <t>OLIDEN 55</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>811627070</t>
+          <t>814107070</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2535,17 +2535,17 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L25" t="n">
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.490765</v>
+        <v>-58.517269</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.627337</v>
+        <v>-34.639879</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>DEV-I</t>
+          <t>PAV-B</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2571,22 +2571,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8481</t>
+          <t>8882</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>3/18/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CISNEROS, VIRREY 1610</t>
+          <t>EL PROFETA DE LA PAMPA 4523</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>812440520</t>
+          <t>812879773</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2616,26 +2616,26 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.469727</v>
+        <v>-58.477211</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.612013</v>
+        <v>-34.652708</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>PAV-O</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2657,17 +2657,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>8554</t>
+          <t>00239146</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>3/9/2026</t>
+          <t>3/19/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>OLIDEN 55</t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>814107070</t>
+          <t>812879780</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2714,10 +2714,10 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.517269</v>
+        <v>-58.50158</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.639879</v>
+        <v>-34.648954</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>PAV-B</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2743,22 +2743,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>8882</t>
+          <t xml:space="preserve">7460 </t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>3/18/2026</t>
+          <t>3/21/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EL PROFETA DE LA PAMPA 4523</t>
+          <t>TERRADA 2720</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>812879773</t>
+          <t>812879976</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2778,36 +2778,36 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>RIENDA A PIQUE CORTADA</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.477211</v>
+        <v>-58.486103</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.652708</v>
+        <v>-34.603895</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>PAV-O</t>
+          <t>NRA-P</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2829,17 +2829,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>00239146</t>
+          <t>S00463265</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>3/19/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>812879780</t>
+          <t>813353208</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2879,17 +2879,17 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.50158</v>
+        <v>-58.508425</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.648954</v>
+        <v>-34.653353</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2915,17 +2915,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">7460 </t>
+          <t xml:space="preserve">900009976210 </t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>3/21/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TERRADA 2720</t>
+          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>812879976</t>
+          <t>814109781</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2950,12 +2950,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>RIENDA A PIQUE CORTADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2965,17 +2965,17 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.486103</v>
+        <v>-58.477456</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.603895</v>
+        <v>-34.614971</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>NRA-P</t>
+          <t>NRA-M</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3001,22 +3001,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>S00400580</t>
+          <t xml:space="preserve">8734 </t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>4/14/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BORDABEHERE, ENZO 2802</t>
+          <t>ARISMENDI 2916</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>813304660</t>
+          <t>814108006</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE DE MADERA POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3058,10 +3058,10 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.480405</v>
+        <v>-58.479126</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.600087</v>
+        <v>-34.586673</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>PUE-A</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3087,22 +3087,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9022</t>
+          <t xml:space="preserve">10037 </t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGARIÑOS CERVANTES, A. 2072 </t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>813352594</t>
+          <t>814108096</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3137,21 +3137,21 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.46936</v>
+        <v>-58.50158</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.60805</v>
+        <v>-34.648954</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>NRA-K</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3173,17 +3173,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>S00463265</t>
+          <t xml:space="preserve">10058 </t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
+          <t xml:space="preserve">OLIDEN 1187 </t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>813353208</t>
+          <t>814111720</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3230,10 +3230,10 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.508425</v>
+        <v>-58.507509</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.653353</v>
+        <v>-34.650225</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3259,22 +3259,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">9139 </t>
+          <t xml:space="preserve">10151 </t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MOSCONI GENERAL AV. 3327</t>
+          <t>LAGUNA 1562</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>814108508</t>
+          <t>814111819</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3309,21 +3309,21 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.508028</v>
+        <v>-58.467824</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.589722</v>
+        <v>-34.649072</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>PUE-N</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3345,22 +3345,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009976210 </t>
+          <t>-784</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
+          <t>PERON, EVA AV. 7255</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>814109781</t>
+          <t>814125579</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3402,14 +3402,14 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.477456</v>
+        <v>-58.499701</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.614971</v>
+        <v>-34.672846</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>NRA-M</t>
+          <t>PAV-K</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3431,22 +3431,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">8734 </t>
+          <t>-795</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ARISMENDI 2916</t>
+          <t>CABEZON, JOSE LEON 3494</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>814108006</t>
+          <t>814125617</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>base podrida</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3488,10 +3488,10 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.479126</v>
+        <v>-58.51297</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.586673</v>
+        <v>-34.587773</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3517,22 +3517,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">10037 </t>
+          <t>-812</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>MURATURE 4536</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>814108096</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3562,22 +3562,22 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.50158</v>
+        <v>-58.496245</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.648954</v>
+        <v>-34.625987</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>DEV-I</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3603,17 +3603,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">10058 </t>
+          <t>-821</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">OLIDEN 1187 </t>
+          <t>PIZARRO 7485</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>814111720</t>
+          <t>814125705</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3660,10 +3660,10 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.507509</v>
+        <v>-58.518126</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.650225</v>
+        <v>-34.658739</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3681,608 +3681,6 @@
         </is>
       </c>
       <c r="R38" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10073 </t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>GUALEGUAYCHU 3464</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>814111762</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>COLUMNA INCLINADA</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L39" t="n">
-        <v>1</v>
-      </c>
-      <c r="M39" t="n">
-        <v>-58.511499</v>
-      </c>
-      <c r="N39" t="n">
-        <v>-34.603949</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>DEV-C</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10151 </t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>LAGUNA 1562</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>814111819</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>COLUMNA INCLINADA</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="L40" t="n">
-        <v>1</v>
-      </c>
-      <c r="M40" t="n">
-        <v>-58.467824</v>
-      </c>
-      <c r="N40" t="n">
-        <v>-34.649072</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>PPT-N</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>-784</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>PERON, EVA AV. 7255</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>814125579</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L41" t="n">
-        <v>1</v>
-      </c>
-      <c r="M41" t="n">
-        <v>-58.499701</v>
-      </c>
-      <c r="N41" t="n">
-        <v>-34.672846</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>PAV-K</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>-795</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>CABEZON, JOSE LEON 3494</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>814125617</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>base podrida</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L42" t="n">
-        <v>1</v>
-      </c>
-      <c r="M42" t="n">
-        <v>-58.51297</v>
-      </c>
-      <c r="N42" t="n">
-        <v>-34.587773</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>PUE-J</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>-812</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>MURATURE 4536</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L43" t="n">
-        <v>1</v>
-      </c>
-      <c r="M43" t="n">
-        <v>-58.496245</v>
-      </c>
-      <c r="N43" t="n">
-        <v>-34.625987</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>DEV-I</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>-817</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>CISNEROS, VIRREY 1699</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>814125680</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>podrida en base</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L44" t="n">
-        <v>1</v>
-      </c>
-      <c r="M44" t="n">
-        <v>-58.470179</v>
-      </c>
-      <c r="N44" t="n">
-        <v>-34.611301</v>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>NRA-K</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>-821</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>6/2/2026</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>PIZARRO 7485</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>814125705</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>inclinada</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L45" t="n">
-        <v>1</v>
-      </c>
-      <c r="M45" t="n">
-        <v>-58.518126</v>
-      </c>
-      <c r="N45" t="n">
-        <v>-34.658739</v>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>PAV-I</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-28 09:49:59)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R207"/>
+  <dimension ref="A1:R208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18164,6 +18164,92 @@
         </is>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>814703095</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>6/27/2026</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>MAGARIÑOS CERVANTES 2058</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>814703095</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L208" t="n">
+        <v>1</v>
+      </c>
+      <c r="M208" t="n">
+        <v>-58.46936</v>
+      </c>
+      <c r="N208" t="n">
+        <v>-34.60805</v>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>NRA-K</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-28 12:17:10)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R208"/>
+  <dimension ref="A1:R207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12425,7 +12425,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>8779</t>
+          <t>8803</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>NAON ROMULO 3405</t>
+          <t>BARZANA 1685</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -12450,7 +12450,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>813046635</t>
+          <t>813046666</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -12460,12 +12460,12 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>APLOMAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -12482,14 +12482,14 @@
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>-58.480063</v>
+        <v>-58.484374</v>
       </c>
       <c r="N141" t="n">
-        <v>-34.558156</v>
+        <v>-34.583484</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
@@ -12499,7 +12499,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>COG-N</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -12511,7 +12511,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>8803</t>
+          <t>8811</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -12521,7 +12521,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>BARZANA 1685</t>
+          <t>ARGERICH 3685</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -12536,7 +12536,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>813046666</t>
+          <t>813046706</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -12551,7 +12551,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
@@ -12568,10 +12568,10 @@
         <v>1</v>
       </c>
       <c r="M142" t="n">
-        <v>-58.484374</v>
+        <v>-58.496794</v>
       </c>
       <c r="N142" t="n">
-        <v>-34.583484</v>
+        <v>-34.594395</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -12585,7 +12585,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>PUE-G</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -12597,7 +12597,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>8811</t>
+          <t>900009925610</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12607,7 +12607,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ARGERICH 3685</t>
+          <t>ASUNCION 3283</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -12622,7 +12622,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>813046706</t>
+          <t>813046810</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -12632,12 +12632,12 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>NORMALIZAR RIENDA A PIQUE</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Tensor</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -12647,17 +12647,17 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L143" t="n">
         <v>1</v>
       </c>
       <c r="M143" t="n">
-        <v>-58.496794</v>
+        <v>-58.501589</v>
       </c>
       <c r="N143" t="n">
-        <v>-34.594395</v>
+        <v>-34.594928</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12683,7 +12683,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>900009925610</t>
+          <t>8840</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>ASUNCION 3283</t>
+          <t>SAN MARTIN AV 6117</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -12708,7 +12708,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>813046810</t>
+          <t>813046903</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -12718,32 +12718,32 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>NORMALIZAR RIENDA A PIQUE</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Tensor</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L144" t="n">
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-58.501589</v>
+        <v>-58.501896</v>
       </c>
       <c r="N144" t="n">
-        <v>-34.594928</v>
+        <v>-34.594873</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12769,7 +12769,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>8840</t>
+          <t>8866</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -12779,7 +12779,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>SAN MARTIN AV 6117</t>
+          <t>ALVAREZ JULIAN 886</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -12794,7 +12794,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>813046903</t>
+          <t>813047047</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -12814,7 +12814,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -12826,24 +12826,24 @@
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>-58.501896</v>
+        <v>-58.43109</v>
       </c>
       <c r="N145" t="n">
-        <v>-34.594873</v>
+        <v>-34.597375</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>PUE-G</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12855,7 +12855,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>8866</t>
+          <t>8868</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -12865,7 +12865,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>ALVAREZ JULIAN 886</t>
+          <t>AV CORRIENTES 5652</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -12880,7 +12880,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>813047047</t>
+          <t>813047446</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -12912,24 +12912,24 @@
         <v>1</v>
       </c>
       <c r="M146" t="n">
-        <v>-58.43109</v>
+        <v>-58.443037</v>
       </c>
       <c r="N146" t="n">
-        <v>-34.597375</v>
+        <v>-34.596062</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>VCR-J</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -12941,7 +12941,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>8868</t>
+          <t>8869</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -12951,7 +12951,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>AV CORRIENTES 5652</t>
+          <t>AV CORRIENTES 5874</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -12966,7 +12966,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>813047446</t>
+          <t>813047486</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -12998,10 +12998,10 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>-58.443037</v>
+        <v>-58.444912</v>
       </c>
       <c r="N147" t="n">
-        <v>-34.596062</v>
+        <v>-34.594319</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -13015,7 +13015,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -13027,7 +13027,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>8869</t>
+          <t>S00349916</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>AV CORRIENTES 5874</t>
+          <t>AGUIRRE 790</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>813047486</t>
+          <t>813047582</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA REMPLAZA CASO 8615</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -13084,24 +13084,24 @@
         <v>1</v>
       </c>
       <c r="M148" t="n">
-        <v>-58.444912</v>
+        <v>-58.438069</v>
       </c>
       <c r="N148" t="n">
-        <v>-34.594319</v>
+        <v>-34.595162</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13113,7 +13113,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>S00349916</t>
+          <t>S00387634</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -13123,7 +13123,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>AGUIRRE 790</t>
+          <t>AV WARNES 339</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>813047582</t>
+          <t>813047693</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA REMPLAZA CASO 8615</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -13170,24 +13170,24 @@
         <v>1</v>
       </c>
       <c r="M149" t="n">
-        <v>-58.438069</v>
+        <v>-58.441925</v>
       </c>
       <c r="N149" t="n">
-        <v>-34.595162</v>
+        <v>-34.602367</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>ALM-N</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13199,17 +13199,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>S00387634</t>
+          <t>S00396906</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>4/11/2026</t>
+          <t>4/14/2026</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>AV WARNES 339</t>
+          <t>MARSELLA 2546</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -13224,7 +13224,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>813047693</t>
+          <t>813304461</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -13256,10 +13256,10 @@
         <v>1</v>
       </c>
       <c r="M150" t="n">
-        <v>-58.441925</v>
+        <v>-58.477848</v>
       </c>
       <c r="N150" t="n">
-        <v>-34.602367</v>
+        <v>-34.582559</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -13273,7 +13273,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>ALM-N</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13285,17 +13285,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>S00396906</t>
+          <t xml:space="preserve">8879 </t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>4/14/2026</t>
+          <t>4/20/2026</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>MARSELLA 2546</t>
+          <t>ALVAREZ THOMAS AV. 1270</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -13310,7 +13310,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>813304461</t>
+          <t>813304767</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -13342,14 +13342,14 @@
         <v>1</v>
       </c>
       <c r="M151" t="n">
-        <v>-58.477848</v>
+        <v>-58.459453</v>
       </c>
       <c r="N151" t="n">
-        <v>-34.582559</v>
+        <v>-34.57843</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P151" t="inlineStr">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>ATH-O</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -13371,7 +13371,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">8879 </t>
+          <t>AL25250</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -13381,7 +13381,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>ALVAREZ THOMAS AV. 1270</t>
+          <t>ARENAL, CONCEPCION 3526</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>813304767</t>
+          <t>813304930</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -13416,7 +13416,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -13428,10 +13428,10 @@
         <v>1</v>
       </c>
       <c r="M152" t="n">
-        <v>-58.459453</v>
+        <v>-58.446573</v>
       </c>
       <c r="N152" t="n">
-        <v>-34.57843</v>
+        <v>-34.5842</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -13445,7 +13445,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>ATH-O</t>
+          <t>ATH-L</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -13457,7 +13457,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>AL25250</t>
+          <t>8913</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>ARENAL, CONCEPCION 3526</t>
+          <t>AVALOS 162</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>813304930</t>
+          <t>813304971</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -13502,26 +13502,26 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L153" t="n">
         <v>1</v>
       </c>
       <c r="M153" t="n">
-        <v>-58.446573</v>
+        <v>-58.465795</v>
       </c>
       <c r="N153" t="n">
-        <v>-34.5842</v>
+        <v>-34.594702</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P153" t="inlineStr">
@@ -13531,7 +13531,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>ATH-L</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -13543,7 +13543,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>8913</t>
+          <t>8914</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -13553,7 +13553,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>AVALOS 162</t>
+          <t>HEREDIA 1301</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -13568,7 +13568,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>813304971</t>
+          <t>813304975</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -13593,21 +13593,21 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L154" t="n">
         <v>1</v>
       </c>
       <c r="M154" t="n">
-        <v>-58.465795</v>
+        <v>-58.463223</v>
       </c>
       <c r="N154" t="n">
-        <v>-34.594702</v>
+        <v>-34.578285</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P154" t="inlineStr">
@@ -13617,7 +13617,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
@@ -13629,7 +13629,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>8914</t>
+          <t>8915</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -13639,7 +13639,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>HEREDIA 1301</t>
+          <t>DE LOS INCAS AV.5475</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -13654,7 +13654,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>813304975</t>
+          <t>813304986</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -13686,14 +13686,14 @@
         <v>1</v>
       </c>
       <c r="M155" t="n">
-        <v>-58.463223</v>
+        <v>-58.484335</v>
       </c>
       <c r="N155" t="n">
-        <v>-34.578285</v>
+        <v>-34.588747</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P155" t="inlineStr">
@@ -13703,7 +13703,7 @@
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
@@ -13715,7 +13715,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>8915</t>
+          <t>8916</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -13725,7 +13725,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>DE LOS INCAS AV.5475</t>
+          <t>GUTENBERG 3097</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -13740,7 +13740,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>813304986</t>
+          <t>813304988</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -13772,10 +13772,10 @@
         <v>1</v>
       </c>
       <c r="M156" t="n">
-        <v>-58.484335</v>
+        <v>-58.499318</v>
       </c>
       <c r="N156" t="n">
-        <v>-34.588747</v>
+        <v>-34.593795</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -13789,7 +13789,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>PUE-Q</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -13801,17 +13801,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>8916</t>
+          <t>8985</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/21/2026</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>GUTENBERG 3097</t>
+          <t>MAURE 4090</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -13826,7 +13826,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>813304988</t>
+          <t>813350809</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -13858,14 +13858,14 @@
         <v>1</v>
       </c>
       <c r="M157" t="n">
-        <v>-58.499318</v>
+        <v>-58.45208</v>
       </c>
       <c r="N157" t="n">
-        <v>-34.593795</v>
+        <v>-34.586988</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P157" t="inlineStr">
@@ -13875,7 +13875,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>PUE-Q</t>
+          <t>ATH-L</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -13887,17 +13887,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>8985</t>
+          <t>S00462787</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>4/21/2026</t>
+          <t>4/24/2026</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>MAURE 4090</t>
+          <t xml:space="preserve">ASUNCION 3089 </t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -13912,7 +13912,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>813350809</t>
+          <t>813353193</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -13922,7 +13922,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR POSTE POR COLUMNA</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -13944,14 +13944,14 @@
         <v>1</v>
       </c>
       <c r="M158" t="n">
-        <v>-58.45208</v>
+        <v>-58.499328</v>
       </c>
       <c r="N158" t="n">
-        <v>-34.586988</v>
+        <v>-34.593529</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P158" t="inlineStr">
@@ -13961,7 +13961,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>ATH-L</t>
+          <t>PUE-Q</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
@@ -13973,7 +13973,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>S00462787</t>
+          <t>S00463265</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -13983,12 +13983,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t xml:space="preserve">ASUNCION 3089 </t>
+          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -13998,7 +13998,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>813353193</t>
+          <t>813353208</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -14008,7 +14008,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>CAMBIAR POSTE POR COLUMNA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -14030,14 +14030,14 @@
         <v>1</v>
       </c>
       <c r="M159" t="n">
-        <v>-58.499328</v>
+        <v>-58.508425</v>
       </c>
       <c r="N159" t="n">
-        <v>-34.593529</v>
+        <v>-34.653353</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P159" t="inlineStr">
@@ -14047,7 +14047,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>PUE-Q</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
@@ -14059,22 +14059,22 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>S00463265</t>
+          <t>GG000026</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>5/1/2026</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>GARCIA GRANDE DE ZEQUEIRA, SEVERO 6488</t>
+          <t>HUSARES 1516</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -14084,7 +14084,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>813353208</t>
+          <t>SE GENERA OT POR PEX</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -14113,27 +14113,23 @@
         </is>
       </c>
       <c r="L160" t="n">
-        <v>1</v>
-      </c>
-      <c r="M160" t="n">
-        <v>-58.508425</v>
-      </c>
-      <c r="N160" t="n">
-        <v>-34.653353</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M160" t="inlineStr"/>
+      <c r="N160" t="inlineStr"/>
       <c r="O160" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>No clasificado, consultar con mantenimiento</t>
         </is>
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -14145,17 +14141,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GG000026</t>
+          <t>9054</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>5/1/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>HUSARES 1516</t>
+          <t>FRAGA 1886</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -14170,7 +14166,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>SE GENERA OT POR PEX</t>
+          <t>813631412</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -14180,12 +14176,12 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -14199,23 +14195,27 @@
         </is>
       </c>
       <c r="L161" t="n">
-        <v>0</v>
-      </c>
-      <c r="M161" t="inlineStr"/>
-      <c r="N161" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M161" t="n">
+        <v>-58.469257</v>
+      </c>
+      <c r="N161" t="n">
+        <v>-34.582734</v>
+      </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>No clasificado, consultar con mantenimiento</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
@@ -14227,7 +14227,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>9054</t>
+          <t>9057</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>FRAGA 1886</t>
+          <t>AV TRIUNVIRATO 3287</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -14252,7 +14252,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>813631412</t>
+          <t>813631414</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -14262,12 +14262,12 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -14284,10 +14284,10 @@
         <v>1</v>
       </c>
       <c r="M162" t="n">
-        <v>-58.469257</v>
+        <v>-58.468328</v>
       </c>
       <c r="N162" t="n">
-        <v>-34.582734</v>
+        <v>-34.583373</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -14313,7 +14313,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>9057</t>
+          <t>9079</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -14323,7 +14323,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>AV TRIUNVIRATO 3287</t>
+          <t>LUGONES 1708</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -14338,7 +14338,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>813631414</t>
+          <t>813631422</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -14370,10 +14370,10 @@
         <v>1</v>
       </c>
       <c r="M163" t="n">
-        <v>-58.468328</v>
+        <v>-58.474081</v>
       </c>
       <c r="N163" t="n">
-        <v>-34.583373</v>
+        <v>-34.577305</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -14387,7 +14387,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>ATH-J</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -14399,7 +14399,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>9079</t>
+          <t>9052</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -14409,7 +14409,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>LUGONES 1708</t>
+          <t>FRAGA 1820</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -14424,7 +14424,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>813631422</t>
+          <t>813631427</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -14434,12 +14434,12 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -14456,10 +14456,10 @@
         <v>1</v>
       </c>
       <c r="M164" t="n">
-        <v>-58.474081</v>
+        <v>-58.468742</v>
       </c>
       <c r="N164" t="n">
-        <v>-34.577305</v>
+        <v>-34.582749</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -14473,7 +14473,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>ATH-J</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -14485,17 +14485,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>9052</t>
+          <t xml:space="preserve">9091 </t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>FRAGA 1820</t>
+          <t>SCALABRINI ORTIZ, RAUL AV. 1088</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -14510,7 +14510,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>813631427</t>
+          <t>813632428</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -14542,24 +14542,24 @@
         <v>1</v>
       </c>
       <c r="M165" t="n">
-        <v>-58.468742</v>
+        <v>-58.430377</v>
       </c>
       <c r="N165" t="n">
-        <v>-34.582749</v>
+        <v>-34.594393</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>VCR-I</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -14571,7 +14571,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">9091 </t>
+          <t>9095</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>SCALABRINI ORTIZ, RAUL AV. 1088</t>
+          <t>ARGERICH 4039</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -14596,7 +14596,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>813632428</t>
+          <t>813632434</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -14628,24 +14628,24 @@
         <v>1</v>
       </c>
       <c r="M166" t="n">
-        <v>-58.430377</v>
+        <v>-58.49905</v>
       </c>
       <c r="N166" t="n">
-        <v>-34.594393</v>
+        <v>-34.591896</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>VCR-I</t>
+          <t>PUE-G</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -14657,17 +14657,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>9095</t>
+          <t xml:space="preserve">9178 </t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>ARGERICH 4039</t>
+          <t>VERA 311</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -14680,11 +14680,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>813632434</t>
-        </is>
-      </c>
+      <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -14692,46 +14688,46 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L167" t="n">
         <v>1</v>
       </c>
       <c r="M167" t="n">
-        <v>-58.49905</v>
+        <v>-58.436262</v>
       </c>
       <c r="N167" t="n">
-        <v>-34.591896</v>
+        <v>-34.600478</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>PUE-G</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
@@ -14743,7 +14739,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">9178 </t>
+          <t xml:space="preserve">9133 </t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -14753,7 +14749,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>VERA 311</t>
+          <t>ESTOMBA 1191</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -14766,7 +14762,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>814108669</t>
+        </is>
+      </c>
       <c r="G168" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -14784,36 +14784,36 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L168" t="n">
         <v>1</v>
       </c>
       <c r="M168" t="n">
-        <v>-58.436262</v>
+        <v>-58.464637</v>
       </c>
       <c r="N168" t="n">
-        <v>-34.600478</v>
+        <v>-34.579742</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
@@ -14825,7 +14825,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t xml:space="preserve">9133 </t>
+          <t xml:space="preserve">9142 </t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -14835,7 +14835,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>ESTOMBA 1191</t>
+          <t>ESTOMBA 1163</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -14850,7 +14850,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>814108669</t>
+          <t>814108680</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -14882,10 +14882,10 @@
         <v>1</v>
       </c>
       <c r="M169" t="n">
-        <v>-58.464637</v>
+        <v>-58.464649</v>
       </c>
       <c r="N169" t="n">
-        <v>-34.579742</v>
+        <v>-34.580057</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -14911,7 +14911,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t xml:space="preserve">9142 </t>
+          <t xml:space="preserve">9146 </t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ESTOMBA 1163</t>
+          <t>HEREDIA 1158</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -14936,7 +14936,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>814108680</t>
+          <t>814108690</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -14968,10 +14968,10 @@
         <v>1</v>
       </c>
       <c r="M170" t="n">
-        <v>-58.464649</v>
+        <v>-58.463317</v>
       </c>
       <c r="N170" t="n">
-        <v>-34.580057</v>
+        <v>-34.580092</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -14997,7 +14997,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t xml:space="preserve">9146 </t>
+          <t xml:space="preserve">9147 </t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -15007,7 +15007,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>HEREDIA 1158</t>
+          <t>ELCANO AV. 3811</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -15022,7 +15022,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>814108690</t>
+          <t>814108711</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -15054,10 +15054,10 @@
         <v>1</v>
       </c>
       <c r="M171" t="n">
-        <v>-58.463317</v>
+        <v>-58.460612</v>
       </c>
       <c r="N171" t="n">
-        <v>-34.580092</v>
+        <v>-34.580887</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -15083,7 +15083,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t xml:space="preserve">9147 </t>
+          <t xml:space="preserve">9149 </t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>ELCANO AV. 3811</t>
+          <t>GIRIBONE 1301</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -15106,11 +15106,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>814108711</t>
-        </is>
-      </c>
+      <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -15128,7 +15124,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -15140,10 +15136,10 @@
         <v>1</v>
       </c>
       <c r="M172" t="n">
-        <v>-58.460612</v>
+        <v>-58.460784</v>
       </c>
       <c r="N172" t="n">
-        <v>-34.580887</v>
+        <v>-34.579621</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -15169,7 +15165,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t xml:space="preserve">9149 </t>
+          <t xml:space="preserve">9150 </t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -15179,7 +15175,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>GIRIBONE 1301</t>
+          <t>GIRIBONE 1365</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -15192,7 +15188,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>814108720</t>
+        </is>
+      </c>
       <c r="G173" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -15210,7 +15210,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -15222,10 +15222,10 @@
         <v>1</v>
       </c>
       <c r="M173" t="n">
-        <v>-58.460784</v>
+        <v>-58.461208</v>
       </c>
       <c r="N173" t="n">
-        <v>-34.579621</v>
+        <v>-34.579609</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -15251,7 +15251,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t xml:space="preserve">9150 </t>
+          <t>9151</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -15261,7 +15261,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>GIRIBONE 1365</t>
+          <t>CHARLONE 1491</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -15276,7 +15276,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>814108720</t>
+          <t>814108759</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -15308,10 +15308,10 @@
         <v>1</v>
       </c>
       <c r="M174" t="n">
-        <v>-58.461208</v>
+        <v>-58.463072</v>
       </c>
       <c r="N174" t="n">
-        <v>-34.579609</v>
+        <v>-34.58065</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -15337,7 +15337,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>9151</t>
+          <t xml:space="preserve">9192 </t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -15347,7 +15347,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>CHARLONE 1491</t>
+          <t>GANDARA 3184</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -15362,7 +15362,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>814108759</t>
+          <t>814109150</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -15394,14 +15394,14 @@
         <v>1</v>
       </c>
       <c r="M175" t="n">
-        <v>-58.463072</v>
+        <v>-58.484009</v>
       </c>
       <c r="N175" t="n">
-        <v>-34.58065</v>
+        <v>-34.585212</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P175" t="inlineStr">
@@ -15411,7 +15411,7 @@
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>ATH-S</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -15423,7 +15423,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t xml:space="preserve">9192 </t>
+          <t>9191</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -15433,7 +15433,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>GANDARA 3184</t>
+          <t>ALTOLAGUIRRE 1417</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -15448,7 +15448,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>814109150</t>
+          <t>814109153</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -15480,10 +15480,10 @@
         <v>1</v>
       </c>
       <c r="M176" t="n">
-        <v>-58.484009</v>
+        <v>-58.482801</v>
       </c>
       <c r="N176" t="n">
-        <v>-34.585212</v>
+        <v>-34.587072</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -15509,7 +15509,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>9191</t>
+          <t xml:space="preserve">9196 </t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -15519,7 +15519,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>ALTOLAGUIRRE 1417</t>
+          <t>PADILLA 1295</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -15534,7 +15534,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>814109153</t>
+          <t>814109185</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -15566,10 +15566,10 @@
         <v>1</v>
       </c>
       <c r="M177" t="n">
-        <v>-58.482801</v>
+        <v>-58.447848</v>
       </c>
       <c r="N177" t="n">
-        <v>-34.587072</v>
+        <v>-34.595146</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -15583,7 +15583,7 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>ATH-S</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -15595,7 +15595,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t xml:space="preserve">9196 </t>
+          <t xml:space="preserve">9198 </t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -15605,7 +15605,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>PADILLA 1295</t>
+          <t>JUSTO, JUAN B. AV. 2960</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -15620,7 +15620,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>814109185</t>
+          <t>814109216</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -15652,10 +15652,10 @@
         <v>1</v>
       </c>
       <c r="M178" t="n">
-        <v>-58.447848</v>
+        <v>-58.44825</v>
       </c>
       <c r="N178" t="n">
-        <v>-34.595146</v>
+        <v>-34.597626</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -15681,7 +15681,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t xml:space="preserve">9198 </t>
+          <t xml:space="preserve">900009976210 </t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -15691,12 +15691,12 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>JUSTO, JUAN B. AV. 2960</t>
+          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -15706,7 +15706,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>814109216</t>
+          <t>814109781</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -15738,10 +15738,10 @@
         <v>1</v>
       </c>
       <c r="M179" t="n">
-        <v>-58.44825</v>
+        <v>-58.477456</v>
       </c>
       <c r="N179" t="n">
-        <v>-34.597626</v>
+        <v>-34.614971</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -15755,7 +15755,7 @@
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>NRA-M</t>
         </is>
       </c>
       <c r="R179" t="inlineStr">
@@ -15767,22 +15767,22 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t xml:space="preserve">900009976210 </t>
+          <t xml:space="preserve">8734 </t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>ESCALADA DE SAN MARTIN, R. 2829</t>
+          <t>ARISMENDI 2916</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -15792,7 +15792,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>814109781</t>
+          <t>814108006</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -15824,10 +15824,10 @@
         <v>1</v>
       </c>
       <c r="M180" t="n">
-        <v>-58.477456</v>
+        <v>-58.479126</v>
       </c>
       <c r="N180" t="n">
-        <v>-34.614971</v>
+        <v>-34.586673</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -15841,7 +15841,7 @@
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>NRA-M</t>
+          <t>ATH-G</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
@@ -15853,7 +15853,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t xml:space="preserve">8734 </t>
+          <t xml:space="preserve">8804 </t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -15863,12 +15863,12 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>ARISMENDI 2916</t>
+          <t>LOPEZ MERINO, FRANCISCO 3988</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>814108006</t>
+          <t>814108011</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -15910,10 +15910,10 @@
         <v>1</v>
       </c>
       <c r="M181" t="n">
-        <v>-58.479126</v>
+        <v>-58.493486</v>
       </c>
       <c r="N181" t="n">
-        <v>-34.586673</v>
+        <v>-34.589105</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -15927,7 +15927,7 @@
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>ATH-G</t>
+          <t>PUE-G</t>
         </is>
       </c>
       <c r="R181" t="inlineStr">
@@ -15939,7 +15939,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">8804 </t>
+          <t xml:space="preserve">10025 </t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -15949,7 +15949,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>LOPEZ MERINO, FRANCISCO 3988</t>
+          <t>JUSTO, JUAN B. AV. 3073</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -15964,7 +15964,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>814108011</t>
+          <t>814111671</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -15974,7 +15974,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -15996,10 +15996,10 @@
         <v>1</v>
       </c>
       <c r="M182" t="n">
-        <v>-58.493486</v>
+        <v>-58.449604</v>
       </c>
       <c r="N182" t="n">
-        <v>-34.589105</v>
+        <v>-34.598286</v>
       </c>
       <c r="O182" t="inlineStr">
         <is>
@@ -16013,7 +16013,7 @@
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>PUE-G</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R182" t="inlineStr">
@@ -16025,7 +16025,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t xml:space="preserve">10025 </t>
+          <t xml:space="preserve">10028 </t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -16035,7 +16035,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>JUSTO, JUAN B. AV. 3073</t>
+          <t>HUMBOLDT 23</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -16048,11 +16048,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>814111671</t>
-        </is>
-      </c>
+      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -16065,12 +16061,12 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Aplomo</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -16082,10 +16078,10 @@
         <v>1</v>
       </c>
       <c r="M183" t="n">
-        <v>-58.449604</v>
+        <v>-58.452473</v>
       </c>
       <c r="N183" t="n">
-        <v>-34.598286</v>
+        <v>-34.598316</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -16111,7 +16107,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">10028 </t>
+          <t xml:space="preserve">10030 </t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -16121,7 +16117,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>HUMBOLDT 23</t>
+          <t>SUSINI, ANTONIO, CNEL. 2190</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -16134,7 +16130,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>814111692</t>
+        </is>
+      </c>
       <c r="G184" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -16147,12 +16147,12 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Aplomo</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -16164,10 +16164,10 @@
         <v>1</v>
       </c>
       <c r="M184" t="n">
-        <v>-58.452473</v>
+        <v>-58.452997</v>
       </c>
       <c r="N184" t="n">
-        <v>-34.598316</v>
+        <v>-34.597674</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -16193,7 +16193,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t xml:space="preserve">10030 </t>
+          <t xml:space="preserve">9053 </t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -16203,7 +16203,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>SUSINI, ANTONIO, CNEL. 2190</t>
+          <t>FRAGA 1848</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -16218,7 +16218,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>814111692</t>
+          <t>814108072</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -16228,7 +16228,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -16250,14 +16250,14 @@
         <v>1</v>
       </c>
       <c r="M185" t="n">
-        <v>-58.452997</v>
+        <v>-58.468977</v>
       </c>
       <c r="N185" t="n">
-        <v>-34.597674</v>
+        <v>-34.582742</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P185" t="inlineStr">
@@ -16267,7 +16267,7 @@
       </c>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R185" t="inlineStr">
@@ -16279,7 +16279,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">9053 </t>
+          <t xml:space="preserve">10037 </t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -16289,12 +16289,12 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>FRAGA 1848</t>
+          <t>POLA 1104</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -16304,7 +16304,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>814108072</t>
+          <t>814108096</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -16329,21 +16329,21 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L186" t="n">
         <v>1</v>
       </c>
       <c r="M186" t="n">
-        <v>-58.468977</v>
+        <v>-58.50158</v>
       </c>
       <c r="N186" t="n">
-        <v>-34.582742</v>
+        <v>-34.648954</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P186" t="inlineStr">
@@ -16353,7 +16353,7 @@
       </c>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R186" t="inlineStr">
@@ -16365,7 +16365,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t xml:space="preserve">10037 </t>
+          <t>S00527817</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -16375,12 +16375,12 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>POLA 1104</t>
+          <t>TINOGASTA 2561</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -16388,11 +16388,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr">
-        <is>
-          <t>814108096</t>
-        </is>
-      </c>
+      <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -16400,12 +16396,12 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>DESMONTAR POSTE</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>Cambio</t>
+          <t>Desmonte</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
@@ -16415,21 +16411,21 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L187" t="n">
         <v>1</v>
       </c>
       <c r="M187" t="n">
-        <v>-58.50158</v>
+        <v>-58.487709</v>
       </c>
       <c r="N187" t="n">
-        <v>-34.648954</v>
+        <v>-34.595778</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P187" t="inlineStr">
@@ -16439,7 +16435,7 @@
       </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>PUE-A</t>
         </is>
       </c>
       <c r="R187" t="inlineStr">
@@ -16451,7 +16447,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>S00527817</t>
+          <t xml:space="preserve">10049 </t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -16461,7 +16457,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>TINOGASTA 2561</t>
+          <t>HEREDIA 1295</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -16474,7 +16470,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr"/>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>814111714</t>
+        </is>
+      </c>
       <c r="G188" t="inlineStr">
         <is>
           <t>INGEME</t>
@@ -16482,12 +16482,12 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>DESMONTAR POSTE</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Desmonte</t>
+          <t>Cambio</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -16504,14 +16504,14 @@
         <v>1</v>
       </c>
       <c r="M188" t="n">
-        <v>-58.487709</v>
+        <v>-58.463173</v>
       </c>
       <c r="N188" t="n">
-        <v>-34.595778</v>
+        <v>-34.57859</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P188" t="inlineStr">
@@ -16521,7 +16521,7 @@
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>PUE-A</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R188" t="inlineStr">
@@ -16533,7 +16533,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">10049 </t>
+          <t xml:space="preserve">10058 </t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -16543,12 +16543,12 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>HEREDIA 1295</t>
+          <t xml:space="preserve">OLIDEN 1187 </t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -16558,7 +16558,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>814111714</t>
+          <t>814111720</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -16590,14 +16590,14 @@
         <v>1</v>
       </c>
       <c r="M189" t="n">
-        <v>-58.463173</v>
+        <v>-58.507509</v>
       </c>
       <c r="N189" t="n">
-        <v>-34.57859</v>
+        <v>-34.650225</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P189" t="inlineStr">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R189" t="inlineStr">
@@ -16619,7 +16619,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t xml:space="preserve">10058 </t>
+          <t xml:space="preserve">10069 </t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -16629,12 +16629,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t xml:space="preserve">OLIDEN 1187 </t>
+          <t xml:space="preserve">CORDOBA AV. 5387 </t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -16644,7 +16644,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>814111720</t>
+          <t>814111735</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -16676,24 +16676,24 @@
         <v>1</v>
       </c>
       <c r="M190" t="n">
-        <v>-58.507509</v>
+        <v>-58.437815</v>
       </c>
       <c r="N190" t="n">
-        <v>-34.650225</v>
+        <v>-34.589036</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P190" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>PAV-I</t>
+          <t>VCR-I</t>
         </is>
       </c>
       <c r="R190" t="inlineStr">
@@ -16705,7 +16705,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">10069 </t>
+          <t xml:space="preserve">10079 </t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -16715,7 +16715,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t xml:space="preserve">CORDOBA AV. 5387 </t>
+          <t>VILLARROEL 1035</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -16730,7 +16730,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>814111735</t>
+          <t>814111768</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -16762,10 +16762,10 @@
         <v>1</v>
       </c>
       <c r="M191" t="n">
-        <v>-58.437815</v>
+        <v>-58.442939</v>
       </c>
       <c r="N191" t="n">
-        <v>-34.589036</v>
+        <v>-34.594741</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -16779,7 +16779,7 @@
       </c>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>VCR-I</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R191" t="inlineStr">
@@ -16791,7 +16791,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t xml:space="preserve">10079 </t>
+          <t xml:space="preserve">10080 </t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -16801,7 +16801,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>VILLARROEL 1035</t>
+          <t>THAMES 549</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -16816,7 +16816,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>814111768</t>
+          <t>814111773</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -16848,10 +16848,10 @@
         <v>1</v>
       </c>
       <c r="M192" t="n">
-        <v>-58.442939</v>
+        <v>-58.442534</v>
       </c>
       <c r="N192" t="n">
-        <v>-34.594741</v>
+        <v>-34.59499</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -16877,7 +16877,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">10080 </t>
+          <t xml:space="preserve">10081 </t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -16887,7 +16887,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>THAMES 549</t>
+          <t xml:space="preserve">CORRIENTES AV. 5697 </t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>814111773</t>
+          <t>814111776</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -16934,10 +16934,10 @@
         <v>1</v>
       </c>
       <c r="M193" t="n">
-        <v>-58.442534</v>
+        <v>-58.443323</v>
       </c>
       <c r="N193" t="n">
-        <v>-34.59499</v>
+        <v>-34.595549</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -16963,7 +16963,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">10081 </t>
+          <t xml:space="preserve">10087 </t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -16973,7 +16973,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t xml:space="preserve">CORRIENTES AV. 5697 </t>
+          <t>CASTILLO 40</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -16988,7 +16988,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>814111776</t>
+          <t>814108420</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -17020,10 +17020,10 @@
         <v>1</v>
       </c>
       <c r="M194" t="n">
-        <v>-58.443323</v>
+        <v>-58.430621</v>
       </c>
       <c r="N194" t="n">
-        <v>-34.595549</v>
+        <v>-34.599429</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -17037,7 +17037,7 @@
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>CLI-N</t>
         </is>
       </c>
       <c r="R194" t="inlineStr">
@@ -17049,7 +17049,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve">10087 </t>
+          <t xml:space="preserve">10102 </t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -17059,7 +17059,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>CASTILLO 40</t>
+          <t>ELCANO AV. 3950</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -17074,7 +17074,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>814108420</t>
+          <t>814108464</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -17084,7 +17084,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -17106,24 +17106,24 @@
         <v>1</v>
       </c>
       <c r="M195" t="n">
-        <v>-58.430621</v>
+        <v>-58.460457</v>
       </c>
       <c r="N195" t="n">
-        <v>-34.599429</v>
+        <v>-34.582381</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q195" t="inlineStr">
         <is>
-          <t>CLI-N</t>
+          <t>ATH-H</t>
         </is>
       </c>
       <c r="R195" t="inlineStr">
@@ -17135,7 +17135,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">10102 </t>
+          <t xml:space="preserve">10136 </t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -17145,7 +17145,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>ELCANO AV. 3950</t>
+          <t>REPETTO, NICOLAS, DR. 2118</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -17160,7 +17160,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>814108464</t>
+          <t>814108495</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -17170,7 +17170,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -17192,14 +17192,14 @@
         <v>1</v>
       </c>
       <c r="M196" t="n">
-        <v>-58.460457</v>
+        <v>-58.456381</v>
       </c>
       <c r="N196" t="n">
-        <v>-34.582381</v>
+        <v>-34.60076</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P196" t="inlineStr">
@@ -17209,7 +17209,7 @@
       </c>
       <c r="Q196" t="inlineStr">
         <is>
-          <t>ATH-H</t>
+          <t>NRA-G</t>
         </is>
       </c>
       <c r="R196" t="inlineStr">
@@ -17221,7 +17221,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t xml:space="preserve">10136 </t>
+          <t xml:space="preserve">10151 </t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -17231,12 +17231,12 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 2118</t>
+          <t>LAGUNA 1562</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -17246,7 +17246,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>814108495</t>
+          <t>814111819</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -17256,7 +17256,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>COLUMNA INCLINADA</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -17271,21 +17271,21 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L197" t="n">
         <v>1</v>
       </c>
       <c r="M197" t="n">
-        <v>-58.456381</v>
+        <v>-58.467824</v>
       </c>
       <c r="N197" t="n">
-        <v>-34.60076</v>
+        <v>-34.649072</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P197" t="inlineStr">
@@ -17295,7 +17295,7 @@
       </c>
       <c r="Q197" t="inlineStr">
         <is>
-          <t>NRA-G</t>
+          <t>PPT-N</t>
         </is>
       </c>
       <c r="R197" t="inlineStr">
@@ -17307,17 +17307,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t xml:space="preserve">10151 </t>
+          <t>-784</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>5/14/2026</t>
+          <t>6/2/2026</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>LAGUNA 1562</t>
+          <t>PERON, EVA AV. 7255</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -17332,7 +17332,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>814111819</t>
+          <t>814125579</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -17342,7 +17342,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>COLUMNA INCLINADA</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -17357,17 +17357,17 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L198" t="n">
         <v>1</v>
       </c>
       <c r="M198" t="n">
-        <v>-58.467824</v>
+        <v>-58.499701</v>
       </c>
       <c r="N198" t="n">
-        <v>-34.649072</v>
+        <v>-34.672846</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -17381,7 +17381,7 @@
       </c>
       <c r="Q198" t="inlineStr">
         <is>
-          <t>PPT-N</t>
+          <t>PAV-K</t>
         </is>
       </c>
       <c r="R198" t="inlineStr">
@@ -17393,7 +17393,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>-784</t>
+          <t>-785</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -17403,12 +17403,12 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>PERON, EVA AV. 7255</t>
+          <t>FOREST AV. 1167</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -17418,7 +17418,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>814125579</t>
+          <t>814125584</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -17428,7 +17428,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>columna doblada</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -17450,14 +17450,14 @@
         <v>1</v>
       </c>
       <c r="M199" t="n">
-        <v>-58.499701</v>
+        <v>-58.459624</v>
       </c>
       <c r="N199" t="n">
-        <v>-34.672846</v>
+        <v>-34.578831</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P199" t="inlineStr">
@@ -17467,7 +17467,7 @@
       </c>
       <c r="Q199" t="inlineStr">
         <is>
-          <t>PAV-K</t>
+          <t>ATH-O</t>
         </is>
       </c>
       <c r="R199" t="inlineStr">
@@ -17479,7 +17479,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>-785</t>
+          <t>-789</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -17489,7 +17489,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>FOREST AV. 1167</t>
+          <t>BALLIVIAN 2749</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>814125584</t>
+          <t>814125594</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>columna doblada</t>
+          <t>base corroida</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -17536,14 +17536,14 @@
         <v>1</v>
       </c>
       <c r="M200" t="n">
-        <v>-58.459624</v>
+        <v>-58.481306</v>
       </c>
       <c r="N200" t="n">
-        <v>-34.578831</v>
+        <v>-34.581055</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P200" t="inlineStr">
@@ -17553,7 +17553,7 @@
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>ATH-O</t>
+          <t>ATH-D</t>
         </is>
       </c>
       <c r="R200" t="inlineStr">
@@ -17565,7 +17565,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>-789</t>
+          <t>-795</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -17575,12 +17575,12 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>BALLIVIAN 2749</t>
+          <t>CABEZON, JOSE LEON 3494</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -17590,7 +17590,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>814125594</t>
+          <t>814125617</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -17600,7 +17600,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>base corroida</t>
+          <t>base podrida</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -17622,10 +17622,10 @@
         <v>1</v>
       </c>
       <c r="M201" t="n">
-        <v>-58.481306</v>
+        <v>-58.51297</v>
       </c>
       <c r="N201" t="n">
-        <v>-34.581055</v>
+        <v>-34.587773</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="Q201" t="inlineStr">
         <is>
-          <t>ATH-D</t>
+          <t>PUE-J</t>
         </is>
       </c>
       <c r="R201" t="inlineStr">
@@ -17651,7 +17651,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>-795</t>
+          <t>-803</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -17661,12 +17661,12 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>CABEZON, JOSE LEON 3494</t>
+          <t>LA PAMPA 3810</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -17676,7 +17676,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>814125617</t>
+          <t>814125652</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -17686,7 +17686,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>base podrida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -17708,14 +17708,14 @@
         <v>1</v>
       </c>
       <c r="M202" t="n">
-        <v>-58.51297</v>
+        <v>-58.468358</v>
       </c>
       <c r="N202" t="n">
-        <v>-34.587773</v>
+        <v>-34.573132</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P202" t="inlineStr">
@@ -17725,7 +17725,7 @@
       </c>
       <c r="Q202" t="inlineStr">
         <is>
-          <t>PUE-J</t>
+          <t>ATH-A</t>
         </is>
       </c>
       <c r="R202" t="inlineStr">
@@ -17737,7 +17737,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>-803</t>
+          <t>-812</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -17747,12 +17747,12 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>LA PAMPA 3810</t>
+          <t>MURATURE 4536</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -17762,7 +17762,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>814125652</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -17782,7 +17782,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -17794,14 +17794,14 @@
         <v>1</v>
       </c>
       <c r="M203" t="n">
-        <v>-58.468358</v>
+        <v>-58.496245</v>
       </c>
       <c r="N203" t="n">
-        <v>-34.573132</v>
+        <v>-34.625987</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P203" t="inlineStr">
@@ -17811,7 +17811,7 @@
       </c>
       <c r="Q203" t="inlineStr">
         <is>
-          <t>ATH-A</t>
+          <t>DEV-I</t>
         </is>
       </c>
       <c r="R203" t="inlineStr">
@@ -17823,7 +17823,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>-812</t>
+          <t>-813</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -17833,12 +17833,12 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>MURATURE 4536</t>
+          <t>MURILLO 854</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -17848,7 +17848,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>814125670</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -17858,7 +17858,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>bae corroida</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -17868,7 +17868,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -17880,14 +17880,14 @@
         <v>1</v>
       </c>
       <c r="M204" t="n">
-        <v>-58.496245</v>
+        <v>-58.445269</v>
       </c>
       <c r="N204" t="n">
-        <v>-34.625987</v>
+        <v>-34.599357</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P204" t="inlineStr">
@@ -17897,7 +17897,7 @@
       </c>
       <c r="Q204" t="inlineStr">
         <is>
-          <t>DEV-I</t>
+          <t>VCR-?</t>
         </is>
       </c>
       <c r="R204" t="inlineStr">
@@ -17909,7 +17909,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>-813</t>
+          <t>-821</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -17919,12 +17919,12 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>MURILLO 854</t>
+          <t>PIZARRO 7485</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -17934,7 +17934,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>814125670</t>
+          <t>814125705</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -17944,7 +17944,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>bae corroida</t>
+          <t>inclinada</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -17966,14 +17966,14 @@
         <v>1</v>
       </c>
       <c r="M205" t="n">
-        <v>-58.445269</v>
+        <v>-58.518126</v>
       </c>
       <c r="N205" t="n">
-        <v>-34.599357</v>
+        <v>-34.658739</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P205" t="inlineStr">
@@ -17983,7 +17983,7 @@
       </c>
       <c r="Q205" t="inlineStr">
         <is>
-          <t>VCR-?</t>
+          <t>PAV-I</t>
         </is>
       </c>
       <c r="R205" t="inlineStr">
@@ -17995,22 +17995,22 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>-821</t>
+          <t>994PN</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>6/2/2026</t>
+          <t>6/5/2026</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>PIZARRO 7485</t>
+          <t>MARIANO ACHA 994</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -18020,7 +18020,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>814125705</t>
+          <t>814254408</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -18030,7 +18030,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>inclinada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -18052,14 +18052,14 @@
         <v>1</v>
       </c>
       <c r="M206" t="n">
-        <v>-58.518126</v>
+        <v>-58.472091</v>
       </c>
       <c r="N206" t="n">
-        <v>-34.658739</v>
+        <v>-34.583875</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P206" t="inlineStr">
@@ -18069,7 +18069,7 @@
       </c>
       <c r="Q206" t="inlineStr">
         <is>
-          <t>PAV-I</t>
+          <t>ATH-F</t>
         </is>
       </c>
       <c r="R206" t="inlineStr">
@@ -18081,22 +18081,22 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>994PN</t>
+          <t>814703095</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>6/5/2026</t>
+          <t>6/27/2026</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>MARIANO ACHA 994</t>
+          <t>MAGARIÑOS CERVANTES 2058</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -18106,7 +18106,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>814254408</t>
+          <t>814703095</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -18138,14 +18138,14 @@
         <v>1</v>
       </c>
       <c r="M207" t="n">
-        <v>-58.472091</v>
+        <v>-58.46936</v>
       </c>
       <c r="N207" t="n">
-        <v>-34.583875</v>
+        <v>-34.60805</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P207" t="inlineStr">
@@ -18155,96 +18155,10 @@
       </c>
       <c r="Q207" t="inlineStr">
         <is>
-          <t>ATH-F</t>
+          <t>NRA-K</t>
         </is>
       </c>
       <c r="R207" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>814703095</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>6/27/2026</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>MAGARIÑOS CERVANTES 2058</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F208" t="inlineStr">
-        <is>
-          <t>814703095</t>
-        </is>
-      </c>
-      <c r="G208" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="H208" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I208" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J208" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K208" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L208" t="n">
-        <v>1</v>
-      </c>
-      <c r="M208" t="n">
-        <v>-58.46936</v>
-      </c>
-      <c r="N208" t="n">
-        <v>-34.60805</v>
-      </c>
-      <c r="O208" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="P208" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q208" t="inlineStr">
-        <is>
-          <t>NRA-K</t>
-        </is>
-      </c>
-      <c r="R208" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-29 12:39:24)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_INGEME.xlsx
+++ b/mapa_interactivo_INGEME.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R207"/>
+  <dimension ref="A1:R208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18164,6 +18164,88 @@
         </is>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>814779753</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>6/29/2026</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>AV LA PLATA 724</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>814779753</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr"/>
+      <c r="L208" t="n">
+        <v>1</v>
+      </c>
+      <c r="M208" t="n">
+        <v>-58.427308</v>
+      </c>
+      <c r="N208" t="n">
+        <v>-34.623995</v>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>ALM-A</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>